<commit_message>
Cao trình đỉnh đập: kw tra Bảng A2 TCVN 8421:2010; ghi rõ công thức xấp xỉ đồ thị sóng; bỏ công thức thời gian gió thổi không có nguồn
TCVN 8421:2010 cho chiều cao, chu kỳ sóng nước sâu bằng đồ thị (đường bao trên Hình 1). Excel và Word ghi rõ công thức
gh/V2, gτ/V là công thức xấp xỉ đường bao (Krưlốp). Bỏ công thức quy đổi thời gian gió thổi sang đà gió (hệ số 4,03;
1,6 – không có nguồn): với t = 6 giờ, gt/V ≈ 10^4, điều kiện thời gian không khống chế; Excel có ô nhập giá trị đọc
đồ thị. kw tra Bảng A2 (V <= 20 m/s lấy 2,1·10^-6). cao_trinh_dinh.tinh_truong_hop thêm tùy chọn kw_tra_bang (mặc định
giữ cách cũ cho các script khác). Zđ = +78,87 m không đổi; Δh tăng 1 ÷ 2 mm.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FZ7RkEfpZxiJWB6royQwfj
</commit_message>
<xml_diff>
--- a/DATN_HoCaGiay/TAI_VE/CaoTrinhDinhDap_HoCaGiay.xlsx
+++ b/DATN_HoCaGiay/TAI_VE/CaoTrinhDinhDap_HoCaGiay.xlsx
@@ -52,6 +52,8 @@
     <definedName name="K1_lg">SoLieu!$B$72:$G$72</definedName>
     <definedName name="KRUN_x">SoLieu!$B$75:$H$75</definedName>
     <definedName name="KRUN_k">SoLieu!$B$76:$H$76</definedName>
+    <definedName name="KW_V">SoLieu!$B$79:$E$79</definedName>
+    <definedName name="KW_k">SoLieu!$B$80:$E$80</definedName>
     <definedName name="Z_yc">KetQua!$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -60,11 +62,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
-    <numFmt numFmtId="167" formatCode="+0.00;-0.00;0.00"/>
+    <numFmt numFmtId="167" formatCode="0.0E+00"/>
+    <numFmt numFmtId="168" formatCode="+0.00;-0.00;0.00"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -218,7 +221,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -285,6 +288,9 @@
     <xf numFmtId="165" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="167" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -321,7 +327,7 @@
     <xf numFmtId="2" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="168" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -771,7 +777,7 @@
     <row r="8" ht="22" customHeight="1">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Δh = kw·V²·D/(g·H)·cos α ,   kw = 3·10⁻⁷·(1 + 0,3·V)</t>
+          <t>Δh = kw·V²·D/(g·H)·cos α ,   kw tra Bảng A2: V = 20; 30; 40; 50 m/s → kw = 2,1; 3,0; 3,9; 4,8·10⁻⁶</t>
         </is>
       </c>
     </row>
@@ -796,10 +802,10 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="31" customHeight="1">
+    <row r="12" ht="77.5" customHeight="1">
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>•  Sóng nước sâu (H &gt; 0,5λ̄): gh̄/V² và gτ̄/V theo đường bao trên của đồ thị (Hình 1) – tính theo công thức xấp xỉ, với điều kiện đà gió (gD/V²) và điều kiện thời gian gió thổi t = 6 giờ (gt/V), lấy giá trị nhỏ hơn.</t>
+          <t>•  Sóng nước sâu (H &gt; 0,5λ̄): TCVN 8421:2010 cho gh̄/V² và gτ̄/V bằng đồ thị (Hình 1, đường bao trên), tra theo gD/V² (điều kiện đà gió) và gt/V (điều kiện thời gian gió thổi), lấy giá trị nhỏ hơn – tiêu chuẩn không cho công thức. Để Excel tự tính, đường bao theo đà gió được thay bằng công thức xấp xỉ của Krưlốp (hai công thức dòng trên, λ̄ = gτ̄²/(2π) là công thức của tiêu chuẩn) – nên đọc thử đồ thị 1 ÷ 2 điểm để đối chiếu. Với t = 6 giờ, gt/V ≈ 10⁴: sóng gần phát triển hoàn toàn, đồ thị cho gh̄/V² lớn hơn nhiều so với điều kiện đà gió nên điều kiện thời gian không khống chế; ô “theo điều kiện thời gian” ở TinhSong để trống, nhập giá trị đọc đồ thị nếu muốn kiểm tra.</t>
         </is>
       </c>
     </row>
@@ -866,7 +872,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I76"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -2218,6 +2224,51 @@
       </c>
       <c r="H76" s="25" t="n">
         <v>1.95</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="22" t="inlineStr">
+        <is>
+          <t>Hệ số kw tính độ dềnh do gió (Bảng A2; V ≤ 20 m/s lấy 2,1·10⁻⁶ – bảng không có giá trị nhỏ hơn)</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="23" t="inlineStr">
+        <is>
+          <t>V (m/s)</t>
+        </is>
+      </c>
+      <c r="B79" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="C79" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="D79" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="E79" s="24" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="23" t="inlineStr">
+        <is>
+          <t>kw</t>
+        </is>
+      </c>
+      <c r="B80" s="28" t="n">
+        <v>2.1e-06</v>
+      </c>
+      <c r="C80" s="28" t="n">
+        <v>3e-06</v>
+      </c>
+      <c r="D80" s="28" t="n">
+        <v>3.9e-06</v>
+      </c>
+      <c r="E80" s="28" t="n">
+        <v>4.8e-06</v>
       </c>
     </row>
   </sheetData>
@@ -2336,85 +2387,85 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="28" t="inlineStr">
+      <c r="A4" s="29" t="inlineStr">
         <is>
           <t>Mã hướng gió</t>
         </is>
       </c>
       <c r="B4" s="14" t="inlineStr"/>
-      <c r="C4" s="29" t="inlineStr">
+      <c r="C4" s="30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="D4" s="29" t="inlineStr">
+      <c r="D4" s="30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="E4" s="29" t="inlineStr">
+      <c r="E4" s="30" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="F4" s="29" t="inlineStr">
+      <c r="F4" s="30" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="G4" s="29" t="inlineStr">
+      <c r="G4" s="30" t="inlineStr">
         <is>
           <t>NW</t>
         </is>
       </c>
-      <c r="H4" s="29" t="inlineStr">
+      <c r="H4" s="30" t="inlineStr">
         <is>
           <t>NW</t>
         </is>
       </c>
-      <c r="I4" s="30" t="inlineStr"/>
+      <c r="I4" s="31" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="inlineStr">
+      <c r="A5" s="29" t="inlineStr">
         <is>
           <t>Trường hợp (Z1 – MNDBT, gió P = 4%; Z2 – MNLTK, gió P = 50%)</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr"/>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="30" t="inlineStr">
         <is>
           <t>Z1</t>
         </is>
       </c>
-      <c r="D5" s="29" t="inlineStr">
+      <c r="D5" s="30" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="E5" s="29" t="inlineStr">
+      <c r="E5" s="30" t="inlineStr">
         <is>
           <t>Z1</t>
         </is>
       </c>
-      <c r="F5" s="29" t="inlineStr">
+      <c r="F5" s="30" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="G5" s="29" t="inlineStr">
+      <c r="G5" s="30" t="inlineStr">
         <is>
           <t>Z1</t>
         </is>
       </c>
-      <c r="H5" s="29" t="inlineStr">
+      <c r="H5" s="30" t="inlineStr">
         <is>
           <t>Z2</t>
         </is>
       </c>
-      <c r="I5" s="30" t="inlineStr"/>
+      <c r="I5" s="31" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="inlineStr">
+      <c r="A6" s="29" t="inlineStr">
         <is>
           <t>Mực nước tính toán Z</t>
         </is>
@@ -2424,38 +2475,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="32">
         <f>IF(C5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="32">
         <f>IF(D5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="32">
         <f>IF(E5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="F6" s="31">
+      <c r="F6" s="32">
         <f>IF(F5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="G6" s="31">
+      <c r="G6" s="32">
         <f>IF(G5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="H6" s="31">
+      <c r="H6" s="32">
         <f>IF(H5="Z1",MN_DBT,MN_LTK)</f>
         <v/>
       </c>
-      <c r="I6" s="30" t="inlineStr">
+      <c r="I6" s="31" t="inlineStr">
         <is>
           <t>SoLieu mục A</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="A7" s="29" t="inlineStr">
         <is>
           <t>Chiều sâu nước trước đập H</t>
         </is>
@@ -2465,38 +2516,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="32">
         <f>C6-Z_day</f>
         <v/>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="32">
         <f>D6-Z_day</f>
         <v/>
       </c>
-      <c r="E7" s="31">
+      <c r="E7" s="32">
         <f>E6-Z_day</f>
         <v/>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="32">
         <f>F6-Z_day</f>
         <v/>
       </c>
-      <c r="G7" s="31">
+      <c r="G7" s="32">
         <f>G6-Z_day</f>
         <v/>
       </c>
-      <c r="H7" s="31">
+      <c r="H7" s="32">
         <f>H6-Z_day</f>
         <v/>
       </c>
-      <c r="I7" s="30" t="inlineStr">
+      <c r="I7" s="31" t="inlineStr">
         <is>
           <t>H = Z − Z đáy</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+      <c r="A8" s="29" t="inlineStr">
         <is>
           <t>Vận tốc gió trạm Vl</t>
         </is>
@@ -2506,75 +2557,75 @@
           <t>m/s</t>
         </is>
       </c>
-      <c r="C8" s="32">
+      <c r="C8" s="33">
         <f>IF(C5="Z1",INDEX(Gio_V4,MATCH(C4,Gio_ma,0)),INDEX(Gio_V50,MATCH(C4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="D8" s="32">
+      <c r="D8" s="33">
         <f>IF(D5="Z1",INDEX(Gio_V4,MATCH(D4,Gio_ma,0)),INDEX(Gio_V50,MATCH(D4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="E8" s="32">
+      <c r="E8" s="33">
         <f>IF(E5="Z1",INDEX(Gio_V4,MATCH(E4,Gio_ma,0)),INDEX(Gio_V50,MATCH(E4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="F8" s="32">
+      <c r="F8" s="33">
         <f>IF(F5="Z1",INDEX(Gio_V4,MATCH(F4,Gio_ma,0)),INDEX(Gio_V50,MATCH(F4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="G8" s="32">
+      <c r="G8" s="33">
         <f>IF(G5="Z1",INDEX(Gio_V4,MATCH(G4,Gio_ma,0)),INDEX(Gio_V50,MATCH(G4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="H8" s="32">
+      <c r="H8" s="33">
         <f>IF(H5="Z1",INDEX(Gio_V4,MATCH(H4,Gio_ma,0)),INDEX(Gio_V50,MATCH(H4,Gio_ma,0)))</f>
         <v/>
       </c>
-      <c r="I8" s="30" t="inlineStr">
+      <c r="I8" s="31" t="inlineStr">
         <is>
           <t>Gió P = 4% (Z1), P = 50% (Z2) – SoLieu mục E</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="inlineStr">
+      <c r="A9" s="29" t="inlineStr">
         <is>
           <t>Hệ số quy đổi kl</t>
         </is>
       </c>
       <c r="B9" s="14" t="inlineStr"/>
-      <c r="C9" s="33">
+      <c r="C9" s="34">
         <f>IF(C8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(C8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(C8,KL_V,1))+(C8-INDEX(KL_V,MATCH(C8,KL_V,1)))*(INDEX(KL_k,MATCH(C8,KL_V,1)+1)-INDEX(KL_k,MATCH(C8,KL_V,1)))/(INDEX(KL_V,MATCH(C8,KL_V,1)+1)-INDEX(KL_V,MATCH(C8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="D9" s="33">
+      <c r="D9" s="34">
         <f>IF(D8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(D8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(D8,KL_V,1))+(D8-INDEX(KL_V,MATCH(D8,KL_V,1)))*(INDEX(KL_k,MATCH(D8,KL_V,1)+1)-INDEX(KL_k,MATCH(D8,KL_V,1)))/(INDEX(KL_V,MATCH(D8,KL_V,1)+1)-INDEX(KL_V,MATCH(D8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="E9" s="33">
+      <c r="E9" s="34">
         <f>IF(E8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(E8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(E8,KL_V,1))+(E8-INDEX(KL_V,MATCH(E8,KL_V,1)))*(INDEX(KL_k,MATCH(E8,KL_V,1)+1)-INDEX(KL_k,MATCH(E8,KL_V,1)))/(INDEX(KL_V,MATCH(E8,KL_V,1)+1)-INDEX(KL_V,MATCH(E8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="F9" s="33">
+      <c r="F9" s="34">
         <f>IF(F8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(F8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(F8,KL_V,1))+(F8-INDEX(KL_V,MATCH(F8,KL_V,1)))*(INDEX(KL_k,MATCH(F8,KL_V,1)+1)-INDEX(KL_k,MATCH(F8,KL_V,1)))/(INDEX(KL_V,MATCH(F8,KL_V,1)+1)-INDEX(KL_V,MATCH(F8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="G9" s="33">
+      <c r="G9" s="34">
         <f>IF(G8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(G8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(G8,KL_V,1))+(G8-INDEX(KL_V,MATCH(G8,KL_V,1)))*(INDEX(KL_k,MATCH(G8,KL_V,1)+1)-INDEX(KL_k,MATCH(G8,KL_V,1)))/(INDEX(KL_V,MATCH(G8,KL_V,1)+1)-INDEX(KL_V,MATCH(G8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="H9" s="33">
+      <c r="H9" s="34">
         <f>IF(H8&lt;=INDEX(KL_V,1),INDEX(KL_k,1),IF(H8&gt;=INDEX(KL_V,COUNT(KL_V)),INDEX(KL_k,COUNT(KL_V)),INDEX(KL_k,MATCH(H8,KL_V,1))+(H8-INDEX(KL_V,MATCH(H8,KL_V,1)))*(INDEX(KL_k,MATCH(H8,KL_V,1)+1)-INDEX(KL_k,MATCH(H8,KL_V,1)))/(INDEX(KL_V,MATCH(H8,KL_V,1)+1)-INDEX(KL_V,MATCH(H8,KL_V,1)))))</f>
         <v/>
       </c>
-      <c r="I9" s="30" t="inlineStr">
+      <c r="I9" s="31" t="inlineStr">
         <is>
           <t>Bảng A3, địa hình dạng A</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="inlineStr">
+      <c r="A10" s="29" t="inlineStr">
         <is>
           <t>Vận tốc gió tính toán V = Vw</t>
         </is>
@@ -2584,38 +2635,38 @@
           <t>m/s</t>
         </is>
       </c>
-      <c r="C10" s="31">
+      <c r="C10" s="32">
         <f>k_fl*C9*C8</f>
         <v/>
       </c>
-      <c r="D10" s="31">
+      <c r="D10" s="32">
         <f>k_fl*D9*D8</f>
         <v/>
       </c>
-      <c r="E10" s="31">
+      <c r="E10" s="32">
         <f>k_fl*E9*E8</f>
         <v/>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="32">
         <f>k_fl*F9*F8</f>
         <v/>
       </c>
-      <c r="G10" s="31">
+      <c r="G10" s="32">
         <f>k_fl*G9*G8</f>
         <v/>
       </c>
-      <c r="H10" s="31">
+      <c r="H10" s="32">
         <f>k_fl*H9*H8</f>
         <v/>
       </c>
-      <c r="I10" s="30" t="inlineStr">
+      <c r="I10" s="31" t="inlineStr">
         <is>
           <t>Vw = kfl·kl·Vl (A.3.3)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="inlineStr">
+      <c r="A11" s="29" t="inlineStr">
         <is>
           <t>Góc tới α giữa hướng gió và pháp tuyến mái</t>
         </is>
@@ -2625,34 +2676,34 @@
           <t>°</t>
         </is>
       </c>
-      <c r="C11" s="32">
+      <c r="C11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(C4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="D11" s="32">
+      <c r="D11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(D4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="E11" s="32">
+      <c r="E11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(E4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="F11" s="32">
+      <c r="F11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(F4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="G11" s="32">
+      <c r="G11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(G4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="H11" s="32">
+      <c r="H11" s="33">
         <f>ABS(MOD(INDEX(Gio_az,MATCH(H4,Gio_ma,0))-PT_mai+180,360)-180)</f>
         <v/>
       </c>
-      <c r="I11" s="30" t="inlineStr"/>
+      <c r="I11" s="31" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="inlineStr">
+      <c r="A12" s="29" t="inlineStr">
         <is>
           <t>Đà gió D</t>
         </is>
@@ -2686,47 +2737,47 @@
         <f>IF(H5="Z1",D_1,D_2)</f>
         <v/>
       </c>
-      <c r="I12" s="30" t="inlineStr">
+      <c r="I12" s="31" t="inlineStr">
         <is>
           <t>SoLieu mục C</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="inlineStr">
+      <c r="A13" s="29" t="inlineStr">
         <is>
           <t>gD/V²</t>
         </is>
       </c>
       <c r="B13" s="14" t="inlineStr"/>
-      <c r="C13" s="32">
+      <c r="C13" s="33">
         <f>g_*C12/C10^2</f>
         <v/>
       </c>
-      <c r="D13" s="32">
+      <c r="D13" s="33">
         <f>g_*D12/D10^2</f>
         <v/>
       </c>
-      <c r="E13" s="32">
+      <c r="E13" s="33">
         <f>g_*E12/E10^2</f>
         <v/>
       </c>
-      <c r="F13" s="32">
+      <c r="F13" s="33">
         <f>g_*F12/F10^2</f>
         <v/>
       </c>
-      <c r="G13" s="32">
+      <c r="G13" s="33">
         <f>g_*G12/G10^2</f>
         <v/>
       </c>
-      <c r="H13" s="32">
+      <c r="H13" s="33">
         <f>g_*H12/H10^2</f>
         <v/>
       </c>
-      <c r="I13" s="30" t="inlineStr"/>
+      <c r="I13" s="31" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="inlineStr">
+      <c r="A14" s="29" t="inlineStr">
         <is>
           <t>gt/V (t = 6 giờ)</t>
         </is>
@@ -2756,117 +2807,99 @@
         <f>g_*t_gio*3600/H10</f>
         <v/>
       </c>
-      <c r="I14" s="30" t="inlineStr"/>
+      <c r="I14" s="31" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="inlineStr">
-        <is>
-          <t>gh̄/V² theo điều kiện đà gió</t>
+      <c r="A15" s="29" t="inlineStr">
+        <is>
+          <t>gh̄/V² theo điều kiện đà gió (đường bao Hình 1)</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr"/>
-      <c r="C15" s="34">
+      <c r="C15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(C13))^-2)</f>
         <v/>
       </c>
-      <c r="D15" s="34">
+      <c r="D15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(D13))^-2)</f>
         <v/>
       </c>
-      <c r="E15" s="34">
+      <c r="E15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(E13))^-2)</f>
         <v/>
       </c>
-      <c r="F15" s="34">
+      <c r="F15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(F13))^-2)</f>
         <v/>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(G13))^-2)</f>
         <v/>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="35">
         <f>0.16*(1-(1+0.006*SQRT(H13))^-2)</f>
         <v/>
       </c>
-      <c r="I15" s="30" t="inlineStr">
-        <is>
-          <t>0,16·[1 − (1 + 0,006·√(gD/V²))⁻²]</t>
+      <c r="I15" s="31" t="inlineStr">
+        <is>
+          <t>Công thức xấp xỉ đường bao (Krưlốp): 0,16·[1 − (1 + 0,006·√(gD/V²))⁻²]</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="inlineStr">
-        <is>
-          <t>gh̄/V² theo điều kiện thời gian gió thổi</t>
+      <c r="A16" s="29" t="inlineStr">
+        <is>
+          <t>gh̄/V² theo điều kiện thời gian gió thổi – tra Hình 1 với gt/V (không bắt buộc)</t>
         </is>
       </c>
       <c r="B16" s="14" t="inlineStr"/>
-      <c r="C16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((C14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="D16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((D14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="E16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((E14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="F16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((F14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="G16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((G14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="H16" s="34">
-        <f>0.16*(1-(1+0.006*SQRT((H14/4.03)^1.6))^-2)</f>
-        <v/>
-      </c>
-      <c r="I16" s="30" t="inlineStr">
-        <is>
-          <t>Như trên với đà gió tương đương gD/V² = (gt/V / 4,03)^1,6</t>
+      <c r="C16" s="26" t="n"/>
+      <c r="D16" s="26" t="n"/>
+      <c r="E16" s="26" t="n"/>
+      <c r="F16" s="26" t="n"/>
+      <c r="G16" s="26" t="n"/>
+      <c r="H16" s="26" t="n"/>
+      <c r="I16" s="31" t="inlineStr">
+        <is>
+          <t>Để trống: gt/V ≈ 10⁴ – sóng gần phát triển hoàn toàn, không khống chế</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="inlineStr">
+      <c r="A17" s="29" t="inlineStr">
         <is>
           <t>gh̄/V² chọn (giá trị nhỏ hơn)</t>
         </is>
       </c>
       <c r="B17" s="14" t="inlineStr"/>
-      <c r="C17" s="34">
-        <f>MIN(C15,C16)</f>
-        <v/>
-      </c>
-      <c r="D17" s="34">
-        <f>MIN(D15,D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="34">
-        <f>MIN(E15,E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="34">
-        <f>MIN(F15,F16)</f>
-        <v/>
-      </c>
-      <c r="G17" s="34">
-        <f>MIN(G15,G16)</f>
-        <v/>
-      </c>
-      <c r="H17" s="34">
-        <f>MIN(H15,H16)</f>
-        <v/>
-      </c>
-      <c r="I17" s="30" t="inlineStr"/>
+      <c r="C17" s="35">
+        <f>IF(ISNUMBER(C16),MIN(C15,C16),C15)</f>
+        <v/>
+      </c>
+      <c r="D17" s="35">
+        <f>IF(ISNUMBER(D16),MIN(D15,D16),D15)</f>
+        <v/>
+      </c>
+      <c r="E17" s="35">
+        <f>IF(ISNUMBER(E16),MIN(E15,E16),E15)</f>
+        <v/>
+      </c>
+      <c r="F17" s="35">
+        <f>IF(ISNUMBER(F16),MIN(F15,F16),F15)</f>
+        <v/>
+      </c>
+      <c r="G17" s="35">
+        <f>IF(ISNUMBER(G16),MIN(G15,G16),G15)</f>
+        <v/>
+      </c>
+      <c r="H17" s="35">
+        <f>IF(ISNUMBER(H16),MIN(H15,H16),H15)</f>
+        <v/>
+      </c>
+      <c r="I17" s="31" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="inlineStr">
+      <c r="A18" s="29" t="inlineStr">
         <is>
           <t>Chiều cao sóng trung bình h̄</t>
         </is>
@@ -2876,38 +2909,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="34">
         <f>C17*C10^2/g_</f>
         <v/>
       </c>
-      <c r="D18" s="33">
+      <c r="D18" s="34">
         <f>D17*D10^2/g_</f>
         <v/>
       </c>
-      <c r="E18" s="33">
+      <c r="E18" s="34">
         <f>E17*E10^2/g_</f>
         <v/>
       </c>
-      <c r="F18" s="33">
+      <c r="F18" s="34">
         <f>F17*F10^2/g_</f>
         <v/>
       </c>
-      <c r="G18" s="33">
+      <c r="G18" s="34">
         <f>G17*G10^2/g_</f>
         <v/>
       </c>
-      <c r="H18" s="33">
+      <c r="H18" s="34">
         <f>H17*H10^2/g_</f>
         <v/>
       </c>
-      <c r="I18" s="30" t="inlineStr">
+      <c r="I18" s="31" t="inlineStr">
         <is>
           <t>h̄ = (gh̄/V²)·V²/g</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="inlineStr">
+      <c r="A19" s="29" t="inlineStr">
         <is>
           <t>Chu kỳ sóng trung bình τ̄</t>
         </is>
@@ -2917,38 +2950,38 @@
           <t>s</t>
         </is>
       </c>
-      <c r="C19" s="31">
+      <c r="C19" s="32">
         <f>19.1*C17^0.625*C10/g_</f>
         <v/>
       </c>
-      <c r="D19" s="31">
+      <c r="D19" s="32">
         <f>19.1*D17^0.625*D10/g_</f>
         <v/>
       </c>
-      <c r="E19" s="31">
+      <c r="E19" s="32">
         <f>19.1*E17^0.625*E10/g_</f>
         <v/>
       </c>
-      <c r="F19" s="31">
+      <c r="F19" s="32">
         <f>19.1*F17^0.625*F10/g_</f>
         <v/>
       </c>
-      <c r="G19" s="31">
+      <c r="G19" s="32">
         <f>19.1*G17^0.625*G10/g_</f>
         <v/>
       </c>
-      <c r="H19" s="31">
+      <c r="H19" s="32">
         <f>19.1*H17^0.625*H10/g_</f>
         <v/>
       </c>
-      <c r="I19" s="30" t="inlineStr">
-        <is>
-          <t>gτ̄/V = 19,1·(gh̄/V²)^0,625</t>
+      <c r="I19" s="31" t="inlineStr">
+        <is>
+          <t>Xấp xỉ đường bao (Krưlốp): gτ̄/V = 19,1·(gh̄/V²)^0,625</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="inlineStr">
+      <c r="A20" s="29" t="inlineStr">
         <is>
           <t>Bước sóng trung bình λ̄</t>
         </is>
@@ -2958,38 +2991,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C20" s="31">
+      <c r="C20" s="32">
         <f>g_*C19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="D20" s="31">
+      <c r="D20" s="32">
         <f>g_*D19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="E20" s="31">
+      <c r="E20" s="32">
         <f>g_*E19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="F20" s="31">
+      <c r="F20" s="32">
         <f>g_*F19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="G20" s="31">
+      <c r="G20" s="32">
         <f>g_*G19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="H20" s="31">
+      <c r="H20" s="32">
         <f>g_*H19^2/(2*PI())</f>
         <v/>
       </c>
-      <c r="I20" s="30" t="inlineStr">
+      <c r="I20" s="31" t="inlineStr">
         <is>
           <t>λ̄ = g·τ̄²/(2π)</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="inlineStr">
+      <c r="A21" s="29" t="inlineStr">
         <is>
           <t>Kiểm tra sóng nước sâu H &gt; 0,5λ̄</t>
         </is>
@@ -3019,47 +3052,47 @@
         <f>IF(H7&gt;0.5*H20,"Đúng","Sai – xem lại")</f>
         <v/>
       </c>
-      <c r="I21" s="30" t="inlineStr"/>
+      <c r="I21" s="31" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="A22" s="29" t="inlineStr">
         <is>
           <t>Hệ số K1%</t>
         </is>
       </c>
       <c r="B22" s="14" t="inlineStr"/>
-      <c r="C22" s="33">
+      <c r="C22" s="34">
         <f>IF(LOG10(C13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(C13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1))+(LOG10(C13)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="D22" s="33">
+      <c r="D22" s="34">
         <f>IF(LOG10(D13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(D13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1))+(LOG10(D13)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="E22" s="33">
+      <c r="E22" s="34">
         <f>IF(LOG10(E13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(E13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1))+(LOG10(E13)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="F22" s="33">
+      <c r="F22" s="34">
         <f>IF(LOG10(F13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(F13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1))+(LOG10(F13)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="G22" s="33">
+      <c r="G22" s="34">
         <f>IF(LOG10(G13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(G13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1))+(LOG10(G13)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="H22" s="33">
+      <c r="H22" s="34">
         <f>IF(LOG10(H13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(H13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1))+(LOG10(H13)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))))</f>
         <v/>
       </c>
-      <c r="I22" s="30" t="inlineStr">
+      <c r="I22" s="31" t="inlineStr">
         <is>
           <t>Hình 2, theo gD/V²</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Chiều cao sóng h1% = K1%·h̄</t>
         </is>
@@ -3069,289 +3102,289 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C23" s="33">
+      <c r="C23" s="34">
         <f>C22*C18</f>
         <v/>
       </c>
-      <c r="D23" s="33">
+      <c r="D23" s="34">
         <f>D22*D18</f>
         <v/>
       </c>
-      <c r="E23" s="33">
+      <c r="E23" s="34">
         <f>E22*E18</f>
         <v/>
       </c>
-      <c r="F23" s="33">
+      <c r="F23" s="34">
         <f>F22*F18</f>
         <v/>
       </c>
-      <c r="G23" s="33">
+      <c r="G23" s="34">
         <f>G22*G18</f>
         <v/>
       </c>
-      <c r="H23" s="33">
+      <c r="H23" s="34">
         <f>H22*H18</f>
         <v/>
       </c>
-      <c r="I23" s="30" t="inlineStr"/>
+      <c r="I23" s="31" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>Độ nhám tương đối Δ/h1%</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr"/>
-      <c r="C24" s="34">
+      <c r="C24" s="35">
         <f>Delta_n/C23</f>
         <v/>
       </c>
-      <c r="D24" s="34">
+      <c r="D24" s="35">
         <f>Delta_n/D23</f>
         <v/>
       </c>
-      <c r="E24" s="34">
+      <c r="E24" s="35">
         <f>Delta_n/E23</f>
         <v/>
       </c>
-      <c r="F24" s="34">
+      <c r="F24" s="35">
         <f>Delta_n/F23</f>
         <v/>
       </c>
-      <c r="G24" s="34">
+      <c r="G24" s="35">
         <f>Delta_n/G23</f>
         <v/>
       </c>
-      <c r="H24" s="34">
+      <c r="H24" s="35">
         <f>Delta_n/H23</f>
         <v/>
       </c>
-      <c r="I24" s="30" t="inlineStr">
+      <c r="I24" s="31" t="inlineStr">
         <is>
           <t>Δ = 0,02 m</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>Hệ số nhám kr</t>
         </is>
       </c>
       <c r="B25" s="14" t="inlineStr"/>
-      <c r="C25" s="33">
+      <c r="C25" s="34">
         <f>IF(C24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(C24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(C24,KR_x,1))+(C24-INDEX(KR_x,MATCH(C24,KR_x,1)))*(INDEX(KR_kr,MATCH(C24,KR_x,1)+1)-INDEX(KR_kr,MATCH(C24,KR_x,1)))/(INDEX(KR_x,MATCH(C24,KR_x,1)+1)-INDEX(KR_x,MATCH(C24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="D25" s="33">
+      <c r="D25" s="34">
         <f>IF(D24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(D24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(D24,KR_x,1))+(D24-INDEX(KR_x,MATCH(D24,KR_x,1)))*(INDEX(KR_kr,MATCH(D24,KR_x,1)+1)-INDEX(KR_kr,MATCH(D24,KR_x,1)))/(INDEX(KR_x,MATCH(D24,KR_x,1)+1)-INDEX(KR_x,MATCH(D24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="E25" s="33">
+      <c r="E25" s="34">
         <f>IF(E24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(E24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(E24,KR_x,1))+(E24-INDEX(KR_x,MATCH(E24,KR_x,1)))*(INDEX(KR_kr,MATCH(E24,KR_x,1)+1)-INDEX(KR_kr,MATCH(E24,KR_x,1)))/(INDEX(KR_x,MATCH(E24,KR_x,1)+1)-INDEX(KR_x,MATCH(E24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="F25" s="33">
+      <c r="F25" s="34">
         <f>IF(F24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(F24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(F24,KR_x,1))+(F24-INDEX(KR_x,MATCH(F24,KR_x,1)))*(INDEX(KR_kr,MATCH(F24,KR_x,1)+1)-INDEX(KR_kr,MATCH(F24,KR_x,1)))/(INDEX(KR_x,MATCH(F24,KR_x,1)+1)-INDEX(KR_x,MATCH(F24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="G25" s="33">
+      <c r="G25" s="34">
         <f>IF(G24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(G24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(G24,KR_x,1))+(G24-INDEX(KR_x,MATCH(G24,KR_x,1)))*(INDEX(KR_kr,MATCH(G24,KR_x,1)+1)-INDEX(KR_kr,MATCH(G24,KR_x,1)))/(INDEX(KR_x,MATCH(G24,KR_x,1)+1)-INDEX(KR_x,MATCH(G24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="H25" s="33">
+      <c r="H25" s="34">
         <f>IF(H24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(H24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(H24,KR_x,1))+(H24-INDEX(KR_x,MATCH(H24,KR_x,1)))*(INDEX(KR_kr,MATCH(H24,KR_x,1)+1)-INDEX(KR_kr,MATCH(H24,KR_x,1)))/(INDEX(KR_x,MATCH(H24,KR_x,1)+1)-INDEX(KR_x,MATCH(H24,KR_x,1)))))</f>
         <v/>
       </c>
-      <c r="I25" s="30" t="inlineStr">
+      <c r="I25" s="31" t="inlineStr">
         <is>
           <t>Bảng hệ số nhám, thấm</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>Hệ số thấm kp</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr"/>
-      <c r="C26" s="33">
+      <c r="C26" s="34">
         <f>IF(C24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(C24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(C24,KP_x,1))+(C24-INDEX(KP_x,MATCH(C24,KP_x,1)))*(INDEX(KP_kp,MATCH(C24,KP_x,1)+1)-INDEX(KP_kp,MATCH(C24,KP_x,1)))/(INDEX(KP_x,MATCH(C24,KP_x,1)+1)-INDEX(KP_x,MATCH(C24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="D26" s="33">
+      <c r="D26" s="34">
         <f>IF(D24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(D24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(D24,KP_x,1))+(D24-INDEX(KP_x,MATCH(D24,KP_x,1)))*(INDEX(KP_kp,MATCH(D24,KP_x,1)+1)-INDEX(KP_kp,MATCH(D24,KP_x,1)))/(INDEX(KP_x,MATCH(D24,KP_x,1)+1)-INDEX(KP_x,MATCH(D24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="E26" s="33">
+      <c r="E26" s="34">
         <f>IF(E24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(E24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(E24,KP_x,1))+(E24-INDEX(KP_x,MATCH(E24,KP_x,1)))*(INDEX(KP_kp,MATCH(E24,KP_x,1)+1)-INDEX(KP_kp,MATCH(E24,KP_x,1)))/(INDEX(KP_x,MATCH(E24,KP_x,1)+1)-INDEX(KP_x,MATCH(E24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="F26" s="33">
+      <c r="F26" s="34">
         <f>IF(F24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(F24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(F24,KP_x,1))+(F24-INDEX(KP_x,MATCH(F24,KP_x,1)))*(INDEX(KP_kp,MATCH(F24,KP_x,1)+1)-INDEX(KP_kp,MATCH(F24,KP_x,1)))/(INDEX(KP_x,MATCH(F24,KP_x,1)+1)-INDEX(KP_x,MATCH(F24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="G26" s="33">
+      <c r="G26" s="34">
         <f>IF(G24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(G24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(G24,KP_x,1))+(G24-INDEX(KP_x,MATCH(G24,KP_x,1)))*(INDEX(KP_kp,MATCH(G24,KP_x,1)+1)-INDEX(KP_kp,MATCH(G24,KP_x,1)))/(INDEX(KP_x,MATCH(G24,KP_x,1)+1)-INDEX(KP_x,MATCH(G24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="H26" s="33">
+      <c r="H26" s="34">
         <f>IF(H24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(H24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(H24,KP_x,1))+(H24-INDEX(KP_x,MATCH(H24,KP_x,1)))*(INDEX(KP_kp,MATCH(H24,KP_x,1)+1)-INDEX(KP_kp,MATCH(H24,KP_x,1)))/(INDEX(KP_x,MATCH(H24,KP_x,1)+1)-INDEX(KP_x,MATCH(H24,KP_x,1)))))</f>
         <v/>
       </c>
-      <c r="I26" s="30" t="inlineStr">
+      <c r="I26" s="31" t="inlineStr">
         <is>
           <t>Như trên</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Hệ số ksp</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr"/>
-      <c r="C27" s="33">
+      <c r="C27" s="34">
         <f>IF(C10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(C10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(C10,KSP_V,1))+(C10-INDEX(KSP_V,MATCH(C10,KSP_V,1)))*(INDEX(KSP_k,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(C10,KSP_V,1)))/(INDEX(KSP_V,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(C10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="D27" s="33">
+      <c r="D27" s="34">
         <f>IF(D10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(D10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(D10,KSP_V,1))+(D10-INDEX(KSP_V,MATCH(D10,KSP_V,1)))*(INDEX(KSP_k,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(D10,KSP_V,1)))/(INDEX(KSP_V,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(D10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="E27" s="33">
+      <c r="E27" s="34">
         <f>IF(E10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(E10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(E10,KSP_V,1))+(E10-INDEX(KSP_V,MATCH(E10,KSP_V,1)))*(INDEX(KSP_k,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(E10,KSP_V,1)))/(INDEX(KSP_V,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(E10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="F27" s="33">
+      <c r="F27" s="34">
         <f>IF(F10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(F10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(F10,KSP_V,1))+(F10-INDEX(KSP_V,MATCH(F10,KSP_V,1)))*(INDEX(KSP_k,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(F10,KSP_V,1)))/(INDEX(KSP_V,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(F10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="G27" s="33">
+      <c r="G27" s="34">
         <f>IF(G10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(G10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(G10,KSP_V,1))+(G10-INDEX(KSP_V,MATCH(G10,KSP_V,1)))*(INDEX(KSP_k,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(G10,KSP_V,1)))/(INDEX(KSP_V,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(G10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="H27" s="33">
+      <c r="H27" s="34">
         <f>IF(H10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(H10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(H10,KSP_V,1))+(H10-INDEX(KSP_V,MATCH(H10,KSP_V,1)))*(INDEX(KSP_k,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(H10,KSP_V,1)))/(INDEX(KSP_V,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(H10,KSP_V,1)))))</f>
         <v/>
       </c>
-      <c r="I27" s="30" t="inlineStr">
+      <c r="I27" s="31" t="inlineStr">
         <is>
           <t>Bảng ksp, mái m = 3 ÷ 5</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>Độ thoải sóng λ̄/h1%</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr"/>
-      <c r="C28" s="31">
+      <c r="C28" s="32">
         <f>C20/C23</f>
         <v/>
       </c>
-      <c r="D28" s="31">
+      <c r="D28" s="32">
         <f>D20/D23</f>
         <v/>
       </c>
-      <c r="E28" s="31">
+      <c r="E28" s="32">
         <f>E20/E23</f>
         <v/>
       </c>
-      <c r="F28" s="31">
+      <c r="F28" s="32">
         <f>F20/F23</f>
         <v/>
       </c>
-      <c r="G28" s="31">
+      <c r="G28" s="32">
         <f>G20/G23</f>
         <v/>
       </c>
-      <c r="H28" s="31">
+      <c r="H28" s="32">
         <f>H20/H23</f>
         <v/>
       </c>
-      <c r="I28" s="30" t="inlineStr"/>
+      <c r="I28" s="31" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>Hệ số krun</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr"/>
-      <c r="C29" s="33">
+      <c r="C29" s="34">
         <f>IF(C28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(C28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(C28,KRUN_x,1))+(C28-INDEX(KRUN_x,MATCH(C28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(C28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(C28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(C28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(C28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="D29" s="33">
+      <c r="D29" s="34">
         <f>IF(D28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(D28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(D28,KRUN_x,1))+(D28-INDEX(KRUN_x,MATCH(D28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(D28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(D28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(D28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(D28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="E29" s="33">
+      <c r="E29" s="34">
         <f>IF(E28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(E28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(E28,KRUN_x,1))+(E28-INDEX(KRUN_x,MATCH(E28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(E28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(E28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(E28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(E28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="F29" s="33">
+      <c r="F29" s="34">
         <f>IF(F28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(F28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(F28,KRUN_x,1))+(F28-INDEX(KRUN_x,MATCH(F28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(F28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(F28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(F28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(F28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="G29" s="33">
+      <c r="G29" s="34">
         <f>IF(G28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(G28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(G28,KRUN_x,1))+(G28-INDEX(KRUN_x,MATCH(G28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(G28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(G28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(G28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(G28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="H29" s="33">
+      <c r="H29" s="34">
         <f>IF(H28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(H28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(H28,KRUN_x,1))+(H28-INDEX(KRUN_x,MATCH(H28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(H28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(H28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(H28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(H28,KRUN_x,1)))))</f>
         <v/>
       </c>
-      <c r="I29" s="30" t="inlineStr">
+      <c r="I29" s="31" t="inlineStr">
         <is>
           <t>Hình 10, mái m = 3</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>Hệ số kα</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr"/>
-      <c r="C30" s="33">
+      <c r="C30" s="34">
         <f>IF(C11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(C11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(C11,KA_goc,1))+(C11-INDEX(KA_goc,MATCH(C11,KA_goc,1)))*(INDEX(KA_k,MATCH(C11,KA_goc,1)+1)-INDEX(KA_k,MATCH(C11,KA_goc,1)))/(INDEX(KA_goc,MATCH(C11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(C11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="D30" s="33">
+      <c r="D30" s="34">
         <f>IF(D11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(D11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(D11,KA_goc,1))+(D11-INDEX(KA_goc,MATCH(D11,KA_goc,1)))*(INDEX(KA_k,MATCH(D11,KA_goc,1)+1)-INDEX(KA_k,MATCH(D11,KA_goc,1)))/(INDEX(KA_goc,MATCH(D11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(D11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="E30" s="33">
+      <c r="E30" s="34">
         <f>IF(E11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(E11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(E11,KA_goc,1))+(E11-INDEX(KA_goc,MATCH(E11,KA_goc,1)))*(INDEX(KA_k,MATCH(E11,KA_goc,1)+1)-INDEX(KA_k,MATCH(E11,KA_goc,1)))/(INDEX(KA_goc,MATCH(E11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(E11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="F30" s="33">
+      <c r="F30" s="34">
         <f>IF(F11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(F11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(F11,KA_goc,1))+(F11-INDEX(KA_goc,MATCH(F11,KA_goc,1)))*(INDEX(KA_k,MATCH(F11,KA_goc,1)+1)-INDEX(KA_k,MATCH(F11,KA_goc,1)))/(INDEX(KA_goc,MATCH(F11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(F11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="G30" s="33">
+      <c r="G30" s="34">
         <f>IF(G11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(G11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(G11,KA_goc,1))+(G11-INDEX(KA_goc,MATCH(G11,KA_goc,1)))*(INDEX(KA_k,MATCH(G11,KA_goc,1)+1)-INDEX(KA_k,MATCH(G11,KA_goc,1)))/(INDEX(KA_goc,MATCH(G11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(G11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="H30" s="33">
+      <c r="H30" s="34">
         <f>IF(H11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(H11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(H11,KA_goc,1))+(H11-INDEX(KA_goc,MATCH(H11,KA_goc,1)))*(INDEX(KA_k,MATCH(H11,KA_goc,1)+1)-INDEX(KA_k,MATCH(H11,KA_goc,1)))/(INDEX(KA_goc,MATCH(H11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(H11,KA_goc,1)))))</f>
         <v/>
       </c>
-      <c r="I30" s="30" t="inlineStr">
+      <c r="I30" s="31" t="inlineStr">
         <is>
           <t>Bảng 9, theo α</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="35" t="inlineStr">
+      <c r="A31" s="36" t="inlineStr">
         <is>
           <t>Chiều cao sóng leo hsl1%</t>
         </is>
@@ -3385,51 +3418,51 @@
         <f>H25*H26*H27*H29*H30*H23</f>
         <v/>
       </c>
-      <c r="I31" s="30" t="inlineStr">
+      <c r="I31" s="31" t="inlineStr">
         <is>
           <t>hsl1% = kr·kp·ksp·krun·kα·h1%</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="inlineStr">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>Hệ số kw</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr"/>
-      <c r="C32" s="36">
-        <f>3E-7*(1+0.3*C10)</f>
-        <v/>
-      </c>
-      <c r="D32" s="36">
-        <f>3E-7*(1+0.3*D10)</f>
-        <v/>
-      </c>
-      <c r="E32" s="36">
-        <f>3E-7*(1+0.3*E10)</f>
-        <v/>
-      </c>
-      <c r="F32" s="36">
-        <f>3E-7*(1+0.3*F10)</f>
-        <v/>
-      </c>
-      <c r="G32" s="36">
-        <f>3E-7*(1+0.3*G10)</f>
-        <v/>
-      </c>
-      <c r="H32" s="36">
-        <f>3E-7*(1+0.3*H10)</f>
-        <v/>
-      </c>
-      <c r="I32" s="30" t="inlineStr">
-        <is>
-          <t>kw = 3·10⁻⁷·(1 + 0,3·Vw)</t>
+      <c r="C32" s="37">
+        <f>IF(C10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(C10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(C10,KW_V,1))+(C10-INDEX(KW_V,MATCH(C10,KW_V,1)))*(INDEX(KW_k,MATCH(C10,KW_V,1)+1)-INDEX(KW_k,MATCH(C10,KW_V,1)))/(INDEX(KW_V,MATCH(C10,KW_V,1)+1)-INDEX(KW_V,MATCH(C10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="D32" s="37">
+        <f>IF(D10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(D10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(D10,KW_V,1))+(D10-INDEX(KW_V,MATCH(D10,KW_V,1)))*(INDEX(KW_k,MATCH(D10,KW_V,1)+1)-INDEX(KW_k,MATCH(D10,KW_V,1)))/(INDEX(KW_V,MATCH(D10,KW_V,1)+1)-INDEX(KW_V,MATCH(D10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="E32" s="37">
+        <f>IF(E10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(E10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(E10,KW_V,1))+(E10-INDEX(KW_V,MATCH(E10,KW_V,1)))*(INDEX(KW_k,MATCH(E10,KW_V,1)+1)-INDEX(KW_k,MATCH(E10,KW_V,1)))/(INDEX(KW_V,MATCH(E10,KW_V,1)+1)-INDEX(KW_V,MATCH(E10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="F32" s="37">
+        <f>IF(F10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(F10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(F10,KW_V,1))+(F10-INDEX(KW_V,MATCH(F10,KW_V,1)))*(INDEX(KW_k,MATCH(F10,KW_V,1)+1)-INDEX(KW_k,MATCH(F10,KW_V,1)))/(INDEX(KW_V,MATCH(F10,KW_V,1)+1)-INDEX(KW_V,MATCH(F10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="G32" s="37">
+        <f>IF(G10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(G10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(G10,KW_V,1))+(G10-INDEX(KW_V,MATCH(G10,KW_V,1)))*(INDEX(KW_k,MATCH(G10,KW_V,1)+1)-INDEX(KW_k,MATCH(G10,KW_V,1)))/(INDEX(KW_V,MATCH(G10,KW_V,1)+1)-INDEX(KW_V,MATCH(G10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="H32" s="37">
+        <f>IF(H10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(H10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(H10,KW_V,1))+(H10-INDEX(KW_V,MATCH(H10,KW_V,1)))*(INDEX(KW_k,MATCH(H10,KW_V,1)+1)-INDEX(KW_k,MATCH(H10,KW_V,1)))/(INDEX(KW_V,MATCH(H10,KW_V,1)+1)-INDEX(KW_V,MATCH(H10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="I32" s="31" t="inlineStr">
+        <is>
+          <t>Bảng A2 (V ≤ 20 m/s: 2,1·10⁻⁶)</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="35" t="inlineStr">
+      <c r="A33" s="36" t="inlineStr">
         <is>
           <t>Độ dềnh do gió Δh</t>
         </is>
@@ -3439,38 +3472,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C33" s="37">
+      <c r="C33" s="38">
         <f>C32*C10^2*C12/(g_*C7)*COS(RADIANS(C11))</f>
         <v/>
       </c>
-      <c r="D33" s="37">
+      <c r="D33" s="38">
         <f>D32*D10^2*D12/(g_*D7)*COS(RADIANS(D11))</f>
         <v/>
       </c>
-      <c r="E33" s="37">
+      <c r="E33" s="38">
         <f>E32*E10^2*E12/(g_*E7)*COS(RADIANS(E11))</f>
         <v/>
       </c>
-      <c r="F33" s="37">
+      <c r="F33" s="38">
         <f>F32*F10^2*F12/(g_*F7)*COS(RADIANS(F11))</f>
         <v/>
       </c>
-      <c r="G33" s="37">
+      <c r="G33" s="38">
         <f>G32*G10^2*G12/(g_*G7)*COS(RADIANS(G11))</f>
         <v/>
       </c>
-      <c r="H33" s="37">
+      <c r="H33" s="38">
         <f>H32*H10^2*H12/(g_*H7)*COS(RADIANS(H11))</f>
         <v/>
       </c>
-      <c r="I33" s="30" t="inlineStr">
+      <c r="I33" s="31" t="inlineStr">
         <is>
           <t>Δh = kw·V²·D/(g·H)·cos α</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>Độ vượt cao an toàn</t>
         </is>
@@ -3480,38 +3513,38 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C34" s="31">
+      <c r="C34" s="32">
         <f>IF(C5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="D34" s="31">
+      <c r="D34" s="32">
         <f>IF(D5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="E34" s="31">
+      <c r="E34" s="32">
         <f>IF(E5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="F34" s="31">
+      <c r="F34" s="32">
         <f>IF(F5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="G34" s="31">
+      <c r="G34" s="32">
         <f>IF(G5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="H34" s="31">
+      <c r="H34" s="32">
         <f>IF(H5="Z1",a_1,a_2)</f>
         <v/>
       </c>
-      <c r="I34" s="30" t="inlineStr">
+      <c r="I34" s="31" t="inlineStr">
         <is>
           <t>a (Z1), a′ (Z2) – Bảng 3</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="35" t="inlineStr">
+      <c r="A35" s="36" t="inlineStr">
         <is>
           <t>Cao trình đỉnh đập yêu cầu Z₁ hoặc Z₂</t>
         </is>
@@ -3521,31 +3554,31 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C35" s="38">
+      <c r="C35" s="39">
         <f>C6+C33+C31+C34</f>
         <v/>
       </c>
-      <c r="D35" s="38">
+      <c r="D35" s="39">
         <f>D6+D33+D31+D34</f>
         <v/>
       </c>
-      <c r="E35" s="38">
+      <c r="E35" s="39">
         <f>E6+E33+E31+E34</f>
         <v/>
       </c>
-      <c r="F35" s="38">
+      <c r="F35" s="39">
         <f>F6+F33+F31+F34</f>
         <v/>
       </c>
-      <c r="G35" s="38">
+      <c r="G35" s="39">
         <f>G6+G33+G31+G34</f>
         <v/>
       </c>
-      <c r="H35" s="38">
+      <c r="H35" s="39">
         <f>H6+H33+H31+H34</f>
         <v/>
       </c>
-      <c r="I35" s="30" t="inlineStr">
+      <c r="I35" s="31" t="inlineStr">
         <is>
           <t>Z = Z + Δh + hsl + a</t>
         </is>
@@ -3664,43 +3697,43 @@
           <t>Bắc</t>
         </is>
       </c>
-      <c r="B6" s="32">
+      <c r="B6" s="33">
         <f>TinhSong!C11</f>
         <v/>
       </c>
-      <c r="C6" s="31">
+      <c r="C6" s="32">
         <f>TinhSong!C30</f>
         <v/>
       </c>
-      <c r="D6" s="31">
+      <c r="D6" s="32">
         <f>TinhSong!C10</f>
         <v/>
       </c>
-      <c r="E6" s="31">
+      <c r="E6" s="32">
         <f>TinhSong!D10</f>
         <v/>
       </c>
-      <c r="F6" s="33">
+      <c r="F6" s="34">
         <f>TinhSong!C31</f>
         <v/>
       </c>
-      <c r="G6" s="33">
+      <c r="G6" s="34">
         <f>TinhSong!D31</f>
         <v/>
       </c>
-      <c r="H6" s="39">
+      <c r="H6" s="40">
         <f>TinhSong!C35</f>
         <v/>
       </c>
-      <c r="I6" s="39">
+      <c r="I6" s="40">
         <f>TinhSong!D35</f>
         <v/>
       </c>
-      <c r="J6" s="39">
+      <c r="J6" s="40">
         <f>MN_LKT+a_3</f>
         <v/>
       </c>
-      <c r="K6" s="38">
+      <c r="K6" s="39">
         <f>MAX(H6:J6)</f>
         <v/>
       </c>
@@ -3711,43 +3744,43 @@
           <t>Đông Bắc</t>
         </is>
       </c>
-      <c r="B7" s="32">
+      <c r="B7" s="33">
         <f>TinhSong!E11</f>
         <v/>
       </c>
-      <c r="C7" s="31">
+      <c r="C7" s="32">
         <f>TinhSong!E30</f>
         <v/>
       </c>
-      <c r="D7" s="31">
+      <c r="D7" s="32">
         <f>TinhSong!E10</f>
         <v/>
       </c>
-      <c r="E7" s="31">
+      <c r="E7" s="32">
         <f>TinhSong!F10</f>
         <v/>
       </c>
-      <c r="F7" s="33">
+      <c r="F7" s="34">
         <f>TinhSong!E31</f>
         <v/>
       </c>
-      <c r="G7" s="33">
+      <c r="G7" s="34">
         <f>TinhSong!F31</f>
         <v/>
       </c>
-      <c r="H7" s="39">
+      <c r="H7" s="40">
         <f>TinhSong!E35</f>
         <v/>
       </c>
-      <c r="I7" s="39">
+      <c r="I7" s="40">
         <f>TinhSong!F35</f>
         <v/>
       </c>
-      <c r="J7" s="39">
+      <c r="J7" s="40">
         <f>MN_LKT+a_3</f>
         <v/>
       </c>
-      <c r="K7" s="38">
+      <c r="K7" s="39">
         <f>MAX(H7:J7)</f>
         <v/>
       </c>
@@ -3758,43 +3791,43 @@
           <t>Tây Bắc</t>
         </is>
       </c>
-      <c r="B8" s="32">
+      <c r="B8" s="33">
         <f>TinhSong!G11</f>
         <v/>
       </c>
-      <c r="C8" s="31">
+      <c r="C8" s="32">
         <f>TinhSong!G30</f>
         <v/>
       </c>
-      <c r="D8" s="31">
+      <c r="D8" s="32">
         <f>TinhSong!G10</f>
         <v/>
       </c>
-      <c r="E8" s="31">
+      <c r="E8" s="32">
         <f>TinhSong!H10</f>
         <v/>
       </c>
-      <c r="F8" s="33">
+      <c r="F8" s="34">
         <f>TinhSong!G31</f>
         <v/>
       </c>
-      <c r="G8" s="33">
+      <c r="G8" s="34">
         <f>TinhSong!H31</f>
         <v/>
       </c>
-      <c r="H8" s="39">
+      <c r="H8" s="40">
         <f>TinhSong!G35</f>
         <v/>
       </c>
-      <c r="I8" s="39">
+      <c r="I8" s="40">
         <f>TinhSong!H35</f>
         <v/>
       </c>
-      <c r="J8" s="39">
+      <c r="J8" s="40">
         <f>MN_LKT+a_3</f>
         <v/>
       </c>
-      <c r="K8" s="38">
+      <c r="K8" s="39">
         <f>MAX(H8:J8)</f>
         <v/>
       </c>
@@ -3805,7 +3838,7 @@
           <t>Cao trình đỉnh yêu cầu lớn nhất Zđ (m)</t>
         </is>
       </c>
-      <c r="B9" s="38">
+      <c r="B9" s="39">
         <f>MAX(K6:K8)</f>
         <v/>
       </c>
@@ -3871,106 +3904,106 @@
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
-      <c r="A14" s="35" t="inlineStr">
+      <c r="A14" s="36" t="inlineStr">
         <is>
           <t>Đỉnh tường chắn sóng ≥ Zđ = max(Z₁; Z₂; Z₃)</t>
         </is>
       </c>
-      <c r="B14" s="39">
+      <c r="B14" s="40">
         <f>Z_yc</f>
         <v/>
       </c>
-      <c r="C14" s="31">
+      <c r="C14" s="32">
         <f>Z_tuong</f>
         <v/>
       </c>
-      <c r="D14" s="40">
+      <c r="D14" s="41">
         <f>C14-B14</f>
         <v/>
       </c>
-      <c r="E14" s="41">
+      <c r="E14" s="42">
         <f>IF(D14&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="32">
         <f>Z_tuong</f>
         <v/>
       </c>
-      <c r="G14" s="40">
+      <c r="G14" s="41">
         <f>F14-B14</f>
         <v/>
       </c>
-      <c r="H14" s="41">
+      <c r="H14" s="42">
         <f>IF(G14&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
-      <c r="A15" s="35" t="inlineStr">
+      <c r="A15" s="36" t="inlineStr">
         <is>
           <t>Đỉnh đập không kể tường ≥ MNLKT + 0,3 m</t>
         </is>
       </c>
-      <c r="B15" s="39">
+      <c r="B15" s="40">
         <f>MN_LKT+dZ_LKT</f>
         <v/>
       </c>
-      <c r="C15" s="31">
+      <c r="C15" s="32">
         <f>Z_dinh_HT</f>
         <v/>
       </c>
-      <c r="D15" s="40">
+      <c r="D15" s="41">
         <f>C15-B15</f>
         <v/>
       </c>
-      <c r="E15" s="41">
+      <c r="E15" s="42">
         <f>IF(D15&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="32">
         <f>Z_dinh_SC</f>
         <v/>
       </c>
-      <c r="G15" s="40">
+      <c r="G15" s="41">
         <f>F15-B15</f>
         <v/>
       </c>
-      <c r="H15" s="41">
+      <c r="H15" s="42">
         <f>IF(G15&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="35" t="inlineStr">
+      <c r="A16" s="36" t="inlineStr">
         <is>
           <t>Tường cao hơn đỉnh đập ≤ 1,2 m</t>
         </is>
       </c>
-      <c r="B16" s="39">
+      <c r="B16" s="40">
         <f>dZ_tuong</f>
         <v/>
       </c>
-      <c r="C16" s="31">
+      <c r="C16" s="32">
         <f>Z_tuong-Z_dinh_HT</f>
         <v/>
       </c>
-      <c r="D16" s="40">
+      <c r="D16" s="41">
         <f>B16-C16</f>
         <v/>
       </c>
-      <c r="E16" s="41">
+      <c r="E16" s="42">
         <f>IF(D16&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="32">
         <f>Z_tuong-Z_dinh_SC</f>
         <v/>
       </c>
-      <c r="G16" s="40">
+      <c r="G16" s="41">
         <f>B16-F16</f>
         <v/>
       </c>
-      <c r="H16" s="41">
+      <c r="H16" s="42">
         <f>IF(G16&gt;=-0.0001,"Đạt","Không đạt")</f>
         <v/>
       </c>
@@ -4020,72 +4053,72 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="inlineStr">
+      <c r="A23" s="29" t="inlineStr">
         <is>
           <t>Mực nước tính toán (m)</t>
         </is>
       </c>
-      <c r="B23" s="31">
+      <c r="B23" s="32">
         <f>TinhSong!C6</f>
         <v/>
       </c>
       <c r="C23" s="11" t="n"/>
-      <c r="D23" s="31">
+      <c r="D23" s="32">
         <f>TinhSong!D6</f>
         <v/>
       </c>
       <c r="E23" s="11" t="n"/>
-      <c r="F23" s="31">
+      <c r="F23" s="32">
         <f>MN_LKT</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="inlineStr">
+      <c r="A24" s="29" t="inlineStr">
         <is>
           <t>Vận tốc gió Vl (m/s)</t>
         </is>
       </c>
-      <c r="B24" s="32">
+      <c r="B24" s="33">
         <f>TinhSong!C8</f>
         <v/>
       </c>
       <c r="C24" s="11" t="n"/>
-      <c r="D24" s="32">
+      <c r="D24" s="33">
         <f>TinhSong!D8</f>
         <v/>
       </c>
       <c r="E24" s="11" t="n"/>
-      <c r="F24" s="32" t="inlineStr">
+      <c r="F24" s="33" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="inlineStr">
+      <c r="A25" s="29" t="inlineStr">
         <is>
           <t>Vận tốc gió tính toán Vw (m/s)</t>
         </is>
       </c>
-      <c r="B25" s="31">
+      <c r="B25" s="32">
         <f>TinhSong!C10</f>
         <v/>
       </c>
       <c r="C25" s="11" t="n"/>
-      <c r="D25" s="31">
+      <c r="D25" s="32">
         <f>TinhSong!D10</f>
         <v/>
       </c>
       <c r="E25" s="11" t="n"/>
-      <c r="F25" s="31" t="inlineStr">
+      <c r="F25" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="inlineStr">
+      <c r="A26" s="29" t="inlineStr">
         <is>
           <t>Đà gió D (m)</t>
         </is>
@@ -4107,351 +4140,351 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="inlineStr">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t>Chiều sâu nước trước đập H (m)</t>
         </is>
       </c>
-      <c r="B27" s="31">
+      <c r="B27" s="32">
         <f>TinhSong!C7</f>
         <v/>
       </c>
       <c r="C27" s="11" t="n"/>
-      <c r="D27" s="31">
+      <c r="D27" s="32">
         <f>TinhSong!D7</f>
         <v/>
       </c>
       <c r="E27" s="11" t="n"/>
-      <c r="F27" s="31" t="inlineStr">
+      <c r="F27" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="inlineStr">
+      <c r="A28" s="29" t="inlineStr">
         <is>
           <t>gD/Vw²</t>
         </is>
       </c>
-      <c r="B28" s="32">
+      <c r="B28" s="33">
         <f>TinhSong!C13</f>
         <v/>
       </c>
       <c r="C28" s="11" t="n"/>
-      <c r="D28" s="32">
+      <c r="D28" s="33">
         <f>TinhSong!D13</f>
         <v/>
       </c>
       <c r="E28" s="11" t="n"/>
-      <c r="F28" s="32" t="inlineStr">
+      <c r="F28" s="33" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="inlineStr">
+      <c r="A29" s="29" t="inlineStr">
         <is>
           <t>Chiều cao sóng trung bình h̄ (m)</t>
         </is>
       </c>
-      <c r="B29" s="33">
+      <c r="B29" s="34">
         <f>TinhSong!C18</f>
         <v/>
       </c>
       <c r="C29" s="11" t="n"/>
-      <c r="D29" s="33">
+      <c r="D29" s="34">
         <f>TinhSong!D18</f>
         <v/>
       </c>
       <c r="E29" s="11" t="n"/>
-      <c r="F29" s="33" t="inlineStr">
+      <c r="F29" s="34" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="inlineStr">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t>Chu kỳ τ̄ (s)</t>
         </is>
       </c>
-      <c r="B30" s="31">
+      <c r="B30" s="32">
         <f>TinhSong!C19</f>
         <v/>
       </c>
       <c r="C30" s="11" t="n"/>
-      <c r="D30" s="31">
+      <c r="D30" s="32">
         <f>TinhSong!D19</f>
         <v/>
       </c>
       <c r="E30" s="11" t="n"/>
-      <c r="F30" s="31" t="inlineStr">
+      <c r="F30" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="inlineStr">
+      <c r="A31" s="29" t="inlineStr">
         <is>
           <t>Bước sóng λ̄ (m)</t>
         </is>
       </c>
-      <c r="B31" s="31">
+      <c r="B31" s="32">
         <f>TinhSong!C20</f>
         <v/>
       </c>
       <c r="C31" s="11" t="n"/>
-      <c r="D31" s="31">
+      <c r="D31" s="32">
         <f>TinhSong!D20</f>
         <v/>
       </c>
       <c r="E31" s="11" t="n"/>
-      <c r="F31" s="31" t="inlineStr">
+      <c r="F31" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="inlineStr">
+      <c r="A32" s="29" t="inlineStr">
         <is>
           <t>K1%</t>
         </is>
       </c>
-      <c r="B32" s="31">
+      <c r="B32" s="32">
         <f>TinhSong!C22</f>
         <v/>
       </c>
       <c r="C32" s="11" t="n"/>
-      <c r="D32" s="31">
+      <c r="D32" s="32">
         <f>TinhSong!D22</f>
         <v/>
       </c>
       <c r="E32" s="11" t="n"/>
-      <c r="F32" s="31" t="inlineStr">
+      <c r="F32" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="inlineStr">
+      <c r="A33" s="29" t="inlineStr">
         <is>
           <t>h1% (m)</t>
         </is>
       </c>
-      <c r="B33" s="33">
+      <c r="B33" s="34">
         <f>TinhSong!C23</f>
         <v/>
       </c>
       <c r="C33" s="11" t="n"/>
-      <c r="D33" s="33">
+      <c r="D33" s="34">
         <f>TinhSong!D23</f>
         <v/>
       </c>
       <c r="E33" s="11" t="n"/>
-      <c r="F33" s="33" t="inlineStr">
+      <c r="F33" s="34" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="inlineStr">
+      <c r="A34" s="29" t="inlineStr">
         <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="B34" s="31">
+      <c r="B34" s="32">
         <f>TinhSong!C25</f>
         <v/>
       </c>
       <c r="C34" s="11" t="n"/>
-      <c r="D34" s="31">
+      <c r="D34" s="32">
         <f>TinhSong!D25</f>
         <v/>
       </c>
       <c r="E34" s="11" t="n"/>
-      <c r="F34" s="31" t="inlineStr">
+      <c r="F34" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="28" t="inlineStr">
+      <c r="A35" s="29" t="inlineStr">
         <is>
           <t>kp</t>
         </is>
       </c>
-      <c r="B35" s="31">
+      <c r="B35" s="32">
         <f>TinhSong!C26</f>
         <v/>
       </c>
       <c r="C35" s="11" t="n"/>
-      <c r="D35" s="31">
+      <c r="D35" s="32">
         <f>TinhSong!D26</f>
         <v/>
       </c>
       <c r="E35" s="11" t="n"/>
-      <c r="F35" s="31" t="inlineStr">
+      <c r="F35" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="28" t="inlineStr">
+      <c r="A36" s="29" t="inlineStr">
         <is>
           <t>ksp</t>
         </is>
       </c>
-      <c r="B36" s="31">
+      <c r="B36" s="32">
         <f>TinhSong!C27</f>
         <v/>
       </c>
       <c r="C36" s="11" t="n"/>
-      <c r="D36" s="31">
+      <c r="D36" s="32">
         <f>TinhSong!D27</f>
         <v/>
       </c>
       <c r="E36" s="11" t="n"/>
-      <c r="F36" s="31" t="inlineStr">
+      <c r="F36" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="28" t="inlineStr">
+      <c r="A37" s="29" t="inlineStr">
         <is>
           <t>krun</t>
         </is>
       </c>
-      <c r="B37" s="31">
+      <c r="B37" s="32">
         <f>TinhSong!C29</f>
         <v/>
       </c>
       <c r="C37" s="11" t="n"/>
-      <c r="D37" s="31">
+      <c r="D37" s="32">
         <f>TinhSong!D29</f>
         <v/>
       </c>
       <c r="E37" s="11" t="n"/>
-      <c r="F37" s="31" t="inlineStr">
+      <c r="F37" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="28" t="inlineStr">
+      <c r="A38" s="29" t="inlineStr">
         <is>
           <t>kα</t>
         </is>
       </c>
-      <c r="B38" s="31">
+      <c r="B38" s="32">
         <f>TinhSong!C30</f>
         <v/>
       </c>
       <c r="C38" s="11" t="n"/>
-      <c r="D38" s="31">
+      <c r="D38" s="32">
         <f>TinhSong!D30</f>
         <v/>
       </c>
       <c r="E38" s="11" t="n"/>
-      <c r="F38" s="31" t="inlineStr">
+      <c r="F38" s="32" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="28" t="inlineStr">
+      <c r="A39" s="29" t="inlineStr">
         <is>
           <t>Sóng leo hsl1% (m)</t>
         </is>
       </c>
-      <c r="B39" s="33">
+      <c r="B39" s="34">
         <f>TinhSong!C31</f>
         <v/>
       </c>
       <c r="C39" s="11" t="n"/>
-      <c r="D39" s="33">
+      <c r="D39" s="34">
         <f>TinhSong!D31</f>
         <v/>
       </c>
       <c r="E39" s="11" t="n"/>
-      <c r="F39" s="33" t="inlineStr">
+      <c r="F39" s="34" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="28" t="inlineStr">
+      <c r="A40" s="29" t="inlineStr">
         <is>
           <t>Độ dềnh Δh (m)</t>
         </is>
       </c>
-      <c r="B40" s="33">
+      <c r="B40" s="34">
         <f>TinhSong!C33</f>
         <v/>
       </c>
       <c r="C40" s="11" t="n"/>
-      <c r="D40" s="33">
+      <c r="D40" s="34">
         <f>TinhSong!D33</f>
         <v/>
       </c>
       <c r="E40" s="11" t="n"/>
-      <c r="F40" s="33" t="inlineStr">
+      <c r="F40" s="34" t="inlineStr">
         <is>
           <t>–</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="28" t="inlineStr">
+      <c r="A41" s="29" t="inlineStr">
         <is>
           <t>Độ vượt cao an toàn (m)</t>
         </is>
       </c>
-      <c r="B41" s="31">
+      <c r="B41" s="32">
         <f>TinhSong!C34</f>
         <v/>
       </c>
       <c r="C41" s="11" t="n"/>
-      <c r="D41" s="31">
+      <c r="D41" s="32">
         <f>TinhSong!D34</f>
         <v/>
       </c>
       <c r="E41" s="11" t="n"/>
-      <c r="F41" s="31">
+      <c r="F41" s="32">
         <f>a_3</f>
         <v/>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="35" t="inlineStr">
+      <c r="A42" s="36" t="inlineStr">
         <is>
           <t>Cao trình đỉnh yêu cầu (m)</t>
         </is>
       </c>
-      <c r="B42" s="42">
+      <c r="B42" s="43">
         <f>TinhSong!C35</f>
         <v/>
       </c>
       <c r="C42" s="11" t="n"/>
-      <c r="D42" s="42">
+      <c r="D42" s="43">
         <f>TinhSong!D35</f>
         <v/>
       </c>
       <c r="E42" s="11" t="n"/>
-      <c r="F42" s="42">
+      <c r="F42" s="43">
         <f>MN_LKT+a_3</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Cao trình đỉnh đập: giải thích chiều sâu nước H (đáy lòng hồ +59,0) và hệ số mái m = 3,0 dùng tính sóng leo
H tính từ đáy lòng hồ +59,0 theo bình đồ 2022 (F = 0), không phải đáy đập +54,0 – thiên an toàn cho Δh (lấy +54,0 thì
Δh giảm 1 ÷ 3 mm). Mái thượng lưu m = 3,0 trên cơ +68,0, m = 3,5 dưới cơ: cơ nằm dưới MNDBT 6,70 m, MNLTK 9,43 m, sâu
hơn 0,5λ̄ = 2,9 ÷ 6,4 m nên sóng leo do đoạn m = 3,0 quyết định; Excel thêm dòng kiểm tra, Word thêm hai đoạn giải thích.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FZ7RkEfpZxiJWB6royQwfj
</commit_message>
<xml_diff>
--- a/DATN_HoCaGiay/TAI_VE/CaoTrinhDinhDap_HoCaGiay.xlsx
+++ b/DATN_HoCaGiay/TAI_VE/CaoTrinhDinhDap_HoCaGiay.xlsx
@@ -26,34 +26,35 @@
     <definedName name="D_1">SoLieu!$B$22</definedName>
     <definedName name="D_2">SoLieu!$B$23</definedName>
     <definedName name="m_TL">SoLieu!$B$24</definedName>
-    <definedName name="Delta_n">SoLieu!$B$25</definedName>
-    <definedName name="PT_mai">SoLieu!$B$26</definedName>
-    <definedName name="Z_dinh_HT">SoLieu!$B$30</definedName>
-    <definedName name="Z_tuong">SoLieu!$B$31</definedName>
-    <definedName name="Z_dinh_SC">SoLieu!$B$32</definedName>
-    <definedName name="dZ_LKT">SoLieu!$B$33</definedName>
-    <definedName name="dZ_tuong">SoLieu!$B$34</definedName>
-    <definedName name="Gio_ma">SoLieu!$B$38:$B$45</definedName>
-    <definedName name="Gio_az">SoLieu!$C$38:$C$45</definedName>
-    <definedName name="Gio_V4">SoLieu!$D$38:$D$45</definedName>
-    <definedName name="Gio_V50">SoLieu!$E$38:$E$45</definedName>
-    <definedName name="KL_V">SoLieu!$B$50:$H$50</definedName>
-    <definedName name="KL_k">SoLieu!$B$51:$H$51</definedName>
-    <definedName name="KA_goc">SoLieu!$B$54:$H$54</definedName>
-    <definedName name="KA_k">SoLieu!$B$55:$H$55</definedName>
-    <definedName name="KR_x">SoLieu!$B$58:$G$58</definedName>
-    <definedName name="KR_kr">SoLieu!$B$59:$G$59</definedName>
-    <definedName name="KP_x">SoLieu!$B$62:$G$62</definedName>
-    <definedName name="KP_kp">SoLieu!$B$63:$G$63</definedName>
-    <definedName name="KSP_V">SoLieu!$B$66:$D$66</definedName>
-    <definedName name="KSP_k">SoLieu!$B$67:$D$67</definedName>
-    <definedName name="K1_x">SoLieu!$B$70:$G$70</definedName>
-    <definedName name="K1_k">SoLieu!$B$71:$G$71</definedName>
-    <definedName name="K1_lg">SoLieu!$B$72:$G$72</definedName>
-    <definedName name="KRUN_x">SoLieu!$B$75:$H$75</definedName>
-    <definedName name="KRUN_k">SoLieu!$B$76:$H$76</definedName>
-    <definedName name="KW_V">SoLieu!$B$79:$E$79</definedName>
-    <definedName name="KW_k">SoLieu!$B$80:$E$80</definedName>
+    <definedName name="Z_co_TL">SoLieu!$B$25</definedName>
+    <definedName name="Delta_n">SoLieu!$B$26</definedName>
+    <definedName name="PT_mai">SoLieu!$B$27</definedName>
+    <definedName name="Z_dinh_HT">SoLieu!$B$31</definedName>
+    <definedName name="Z_tuong">SoLieu!$B$32</definedName>
+    <definedName name="Z_dinh_SC">SoLieu!$B$33</definedName>
+    <definedName name="dZ_LKT">SoLieu!$B$34</definedName>
+    <definedName name="dZ_tuong">SoLieu!$B$35</definedName>
+    <definedName name="Gio_ma">SoLieu!$B$39:$B$46</definedName>
+    <definedName name="Gio_az">SoLieu!$C$39:$C$46</definedName>
+    <definedName name="Gio_V4">SoLieu!$D$39:$D$46</definedName>
+    <definedName name="Gio_V50">SoLieu!$E$39:$E$46</definedName>
+    <definedName name="KL_V">SoLieu!$B$51:$H$51</definedName>
+    <definedName name="KL_k">SoLieu!$B$52:$H$52</definedName>
+    <definedName name="KA_goc">SoLieu!$B$55:$H$55</definedName>
+    <definedName name="KA_k">SoLieu!$B$56:$H$56</definedName>
+    <definedName name="KR_x">SoLieu!$B$59:$G$59</definedName>
+    <definedName name="KR_kr">SoLieu!$B$60:$G$60</definedName>
+    <definedName name="KP_x">SoLieu!$B$63:$G$63</definedName>
+    <definedName name="KP_kp">SoLieu!$B$64:$G$64</definedName>
+    <definedName name="KSP_V">SoLieu!$B$67:$D$67</definedName>
+    <definedName name="KSP_k">SoLieu!$B$68:$D$68</definedName>
+    <definedName name="K1_x">SoLieu!$B$71:$G$71</definedName>
+    <definedName name="K1_k">SoLieu!$B$72:$G$72</definedName>
+    <definedName name="K1_lg">SoLieu!$B$73:$G$73</definedName>
+    <definedName name="KRUN_x">SoLieu!$B$76:$H$76</definedName>
+    <definedName name="KRUN_k">SoLieu!$B$77:$H$77</definedName>
+    <definedName name="KW_V">SoLieu!$B$80:$E$80</definedName>
+    <definedName name="KW_k">SoLieu!$B$81:$E$81</definedName>
     <definedName name="Z_yc">KetQua!$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -872,7 +873,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1008,7 +1009,7 @@
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Cao trình đáy hồ trước đập</t>
+          <t>Cao trình đáy lòng hồ trước đập</t>
         </is>
       </c>
       <c r="B9" s="13" t="n">
@@ -1021,7 +1022,7 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Tính chiều sâu nước H = Z − Z đáy (H = 15,70 m ở MNDBT)</t>
+          <t>Bình đồ 2022: F = 0 ở +59,0 (không phải đáy đập +54,0 tính chiều cao đập 24,5 m); H = Z − Z đáy nhỏ hơn → Δh lớn hơn: thiên an toàn</t>
         </is>
       </c>
       <c r="E9" s="10" t="n"/>
@@ -1281,7 +1282,7 @@
     <row r="24">
       <c r="A24" s="12" t="inlineStr">
         <is>
-          <t>Hệ số mái thượng lưu m</t>
+          <t>Hệ số mái thượng lưu m (đoạn trên cơ)</t>
         </is>
       </c>
       <c r="B24" s="17" t="n">
@@ -1290,7 +1291,7 @@
       <c r="C24" s="14" t="inlineStr"/>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>Bảng ksp dưới đây dùng hàng m = 3 ÷ 5</t>
+          <t>Dưới cơ m = 3,5 nằm sâu hơn 0,5λ̄ (TinhSong) – không ảnh hưởng sóng leo; bảng ksp dùng hàng m = 3 ÷ 5</t>
         </is>
       </c>
       <c r="E24" s="10" t="n"/>
@@ -1302,11 +1303,11 @@
     <row r="25">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>Độ nhám lớp gia cố mái Δ</t>
-        </is>
-      </c>
-      <c r="B25" s="18" t="n">
-        <v>0.02</v>
+          <t>Cao trình cơ thượng lưu</t>
+        </is>
+      </c>
+      <c r="B25" s="13" t="n">
+        <v>68</v>
       </c>
       <c r="C25" s="14" t="inlineStr">
         <is>
@@ -1315,7 +1316,7 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Mái gia cố đá xây</t>
+          <t>Thống nhất 21/10/2026</t>
         </is>
       </c>
       <c r="E25" s="10" t="n"/>
@@ -1327,20 +1328,20 @@
     <row r="26">
       <c r="A26" s="12" t="inlineStr">
         <is>
-          <t>Phương vị pháp tuyến mái thượng lưu</t>
-        </is>
-      </c>
-      <c r="B26" s="17" t="n">
-        <v>6.2</v>
+          <t>Độ nhám lớp gia cố mái Δ</t>
+        </is>
+      </c>
+      <c r="B26" s="18" t="n">
+        <v>0.02</v>
       </c>
       <c r="C26" s="14" t="inlineStr">
         <is>
-          <t>°</t>
+          <t>m</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Tuyến đập N96,2°E, lòng hồ phía Bắc</t>
+          <t>Mái gia cố đá xây</t>
         </is>
       </c>
       <c r="E26" s="10" t="n"/>
@@ -1349,57 +1350,57 @@
       <c r="H26" s="10" t="n"/>
       <c r="I26" s="11" t="n"/>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>Phương vị pháp tuyến mái thượng lưu</t>
+        </is>
+      </c>
+      <c r="B27" s="17" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="C27" s="14" t="inlineStr">
+        <is>
+          <t>°</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>Tuyến đập N96,2°E, lòng hồ phía Bắc</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="n"/>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
         <is>
           <t>D. CAO TRÌNH CÔNG TRÌNH (đánh giá theo TCVN 8216:2018 điều 10.1.5)</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t>Thông số</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B30" s="9" t="inlineStr">
         <is>
           <t>Giá trị</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
+      <c r="C30" s="9" t="inlineStr">
         <is>
           <t>Đơn vị</t>
         </is>
       </c>
-      <c r="D29" s="9" t="inlineStr">
+      <c r="D30" s="9" t="inlineStr">
         <is>
           <t>Ghi chú, nguồn</t>
-        </is>
-      </c>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="n"/>
-      <c r="G29" s="10" t="n"/>
-      <c r="H29" s="10" t="n"/>
-      <c r="I29" s="11" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="12" t="inlineStr">
-        <is>
-          <t>Đỉnh đập hiện trạng (hồ sơ thiết kế)</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="n">
-        <v>78.5</v>
-      </c>
-      <c r="C30" s="14" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>Khảo sát đo +78,32 ÷ +78,44 – chỉ để đối chiếu</t>
         </is>
       </c>
       <c r="E30" s="10" t="n"/>
@@ -1411,11 +1412,11 @@
     <row r="31">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Đỉnh tường chắn sóng</t>
+          <t>Đỉnh đập hiện trạng (hồ sơ thiết kế)</t>
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>79.40000000000001</v>
+        <v>78.5</v>
       </c>
       <c r="C31" s="14" t="inlineStr">
         <is>
@@ -1424,7 +1425,7 @@
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>Tường chắn sóng thẳng đứng phía thượng lưu – giữ nguyên</t>
+          <t>Khảo sát đo +78,32 ÷ +78,44 – chỉ để đối chiếu</t>
         </is>
       </c>
       <c r="E31" s="10" t="n"/>
@@ -1436,11 +1437,11 @@
     <row r="32">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Đỉnh đập sau sửa chữa</t>
+          <t>Đỉnh tường chắn sóng</t>
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>78.84999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="C32" s="14" t="inlineStr">
         <is>
@@ -1449,7 +1450,7 @@
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Phương án chọn của đồ án</t>
+          <t>Tường chắn sóng thẳng đứng phía thượng lưu – giữ nguyên</t>
         </is>
       </c>
       <c r="E32" s="10" t="n"/>
@@ -1461,11 +1462,11 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>Đỉnh đập không kể tường cao hơn MNLKT tối thiểu</t>
+          <t>Đỉnh đập sau sửa chữa</t>
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>0.3</v>
+        <v>78.84999999999999</v>
       </c>
       <c r="C33" s="14" t="inlineStr">
         <is>
@@ -1474,7 +1475,7 @@
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>Điều 10.1.5</t>
+          <t>Phương án chọn của đồ án</t>
         </is>
       </c>
       <c r="E33" s="10" t="n"/>
@@ -1486,11 +1487,11 @@
     <row r="34">
       <c r="A34" s="12" t="inlineStr">
         <is>
-          <t>Tường cao hơn đỉnh đập tối đa</t>
+          <t>Đỉnh đập không kể tường cao hơn MNLKT tối thiểu</t>
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>1.2</v>
+        <v>0.3</v>
       </c>
       <c r="C34" s="14" t="inlineStr">
         <is>
@@ -1508,103 +1509,99 @@
       <c r="H34" s="10" t="n"/>
       <c r="I34" s="11" t="n"/>
     </row>
-    <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+    <row r="35">
+      <c r="A35" s="12" t="inlineStr">
+        <is>
+          <t>Tường cao hơn đỉnh đập tối đa</t>
+        </is>
+      </c>
+      <c r="B35" s="13" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="C35" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>Điều 10.1.5</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="10" t="n"/>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="10" t="n"/>
+      <c r="I35" s="11" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr">
         <is>
           <t>E. VẬN TỐC GIÓ LỚN NHẤT THEO HƯỚNG – TRẠM PHAN THIẾT (Bảng 1.4 thuyết minh), m/s</t>
         </is>
       </c>
-      <c r="H36" s="7" t="inlineStr">
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>Tần suất gió theo TCVN 8216:2018 Bảng 4 (cấp II): MNDBT – P = 4%; MNLTK – P = 50% (gió bình quân lớn nhất); MNLKT – không xét sóng.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="32" customHeight="1">
-      <c r="A37" s="9" t="inlineStr">
+    <row r="38" ht="32" customHeight="1">
+      <c r="A38" s="9" t="inlineStr">
         <is>
           <t>Hướng gió</t>
         </is>
       </c>
-      <c r="B37" s="9" t="inlineStr">
+      <c r="B38" s="9" t="inlineStr">
         <is>
           <t>Mã</t>
         </is>
       </c>
-      <c r="C37" s="9" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>Phương vị (°)</t>
         </is>
       </c>
-      <c r="D37" s="9" t="inlineStr">
+      <c r="D38" s="9" t="inlineStr">
         <is>
           <t>V P = 4%</t>
         </is>
       </c>
-      <c r="E37" s="9" t="inlineStr">
+      <c r="E38" s="9" t="inlineStr">
         <is>
           <t>V P = 50%</t>
         </is>
       </c>
-      <c r="F37" s="9" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>Góc tới α (°)</t>
         </is>
       </c>
-      <c r="G37" s="9" t="inlineStr">
+      <c r="G38" s="9" t="inlineStr">
         <is>
           <t>Thổi vào mái TL (α ≤ 60°)?</t>
         </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="12" t="inlineStr">
-        <is>
-          <t>Bắc</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>N</t>
-        </is>
-      </c>
-      <c r="C38" s="19" t="n">
-        <v>0</v>
-      </c>
-      <c r="D38" s="20" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="E38" s="20" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="F38" s="21">
-        <f>ABS(MOD(C38-PT_mai+180,360)-180)</f>
-        <v/>
-      </c>
-      <c r="G38" s="14">
-        <f>IF(F38&lt;=60,"Có – tính","Không")</f>
-        <v/>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Đông Bắc</t>
+          <t>Bắc</t>
         </is>
       </c>
       <c r="B39" s="14" t="inlineStr">
         <is>
-          <t>NE</t>
+          <t>N</t>
         </is>
       </c>
       <c r="C39" s="19" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="D39" s="20" t="n">
-        <v>18.6</v>
+        <v>13.8</v>
       </c>
       <c r="E39" s="20" t="n">
-        <v>11.9</v>
+        <v>7.6</v>
       </c>
       <c r="F39" s="21">
         <f>ABS(MOD(C39-PT_mai+180,360)-180)</f>
@@ -1618,22 +1615,22 @@
     <row r="40">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>Đông</t>
+          <t>Đông Bắc</t>
         </is>
       </c>
       <c r="B40" s="14" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>NE</t>
         </is>
       </c>
       <c r="C40" s="19" t="n">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="D40" s="20" t="n">
-        <v>20.9</v>
+        <v>18.6</v>
       </c>
       <c r="E40" s="20" t="n">
-        <v>15.2</v>
+        <v>11.9</v>
       </c>
       <c r="F40" s="21">
         <f>ABS(MOD(C40-PT_mai+180,360)-180)</f>
@@ -1647,22 +1644,22 @@
     <row r="41">
       <c r="A41" s="12" t="inlineStr">
         <is>
-          <t>Đông Nam</t>
+          <t>Đông</t>
         </is>
       </c>
       <c r="B41" s="14" t="inlineStr">
         <is>
-          <t>SE</t>
+          <t>E</t>
         </is>
       </c>
       <c r="C41" s="19" t="n">
-        <v>135</v>
+        <v>90</v>
       </c>
       <c r="D41" s="20" t="n">
-        <v>15.8</v>
+        <v>20.9</v>
       </c>
       <c r="E41" s="20" t="n">
-        <v>11.4</v>
+        <v>15.2</v>
       </c>
       <c r="F41" s="21">
         <f>ABS(MOD(C41-PT_mai+180,360)-180)</f>
@@ -1676,22 +1673,22 @@
     <row r="42">
       <c r="A42" s="12" t="inlineStr">
         <is>
-          <t>Nam</t>
+          <t>Đông Nam</t>
         </is>
       </c>
       <c r="B42" s="14" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>SE</t>
         </is>
       </c>
       <c r="C42" s="19" t="n">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="D42" s="20" t="n">
-        <v>15.6</v>
+        <v>15.8</v>
       </c>
       <c r="E42" s="20" t="n">
-        <v>11</v>
+        <v>11.4</v>
       </c>
       <c r="F42" s="21">
         <f>ABS(MOD(C42-PT_mai+180,360)-180)</f>
@@ -1705,22 +1702,22 @@
     <row r="43">
       <c r="A43" s="12" t="inlineStr">
         <is>
-          <t>Tây Nam</t>
+          <t>Nam</t>
         </is>
       </c>
       <c r="B43" s="14" t="inlineStr">
         <is>
-          <t>SW</t>
+          <t>S</t>
         </is>
       </c>
       <c r="C43" s="19" t="n">
-        <v>225</v>
+        <v>180</v>
       </c>
       <c r="D43" s="20" t="n">
-        <v>18.9</v>
+        <v>15.6</v>
       </c>
       <c r="E43" s="20" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F43" s="21">
         <f>ABS(MOD(C43-PT_mai+180,360)-180)</f>
@@ -1734,22 +1731,22 @@
     <row r="44">
       <c r="A44" s="12" t="inlineStr">
         <is>
-          <t>Tây</t>
+          <t>Tây Nam</t>
         </is>
       </c>
       <c r="B44" s="14" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>SW</t>
         </is>
       </c>
       <c r="C44" s="19" t="n">
-        <v>270</v>
+        <v>225</v>
       </c>
       <c r="D44" s="20" t="n">
-        <v>20.3</v>
+        <v>18.9</v>
       </c>
       <c r="E44" s="20" t="n">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="F44" s="21">
         <f>ABS(MOD(C44-PT_mai+180,360)-180)</f>
@@ -1763,22 +1760,22 @@
     <row r="45">
       <c r="A45" s="12" t="inlineStr">
         <is>
-          <t>Tây Bắc</t>
+          <t>Tây</t>
         </is>
       </c>
       <c r="B45" s="14" t="inlineStr">
         <is>
-          <t>NW</t>
+          <t>W</t>
         </is>
       </c>
       <c r="C45" s="19" t="n">
-        <v>315</v>
+        <v>270</v>
       </c>
       <c r="D45" s="20" t="n">
-        <v>15.6</v>
+        <v>20.3</v>
       </c>
       <c r="E45" s="20" t="n">
-        <v>8.9</v>
+        <v>14.5</v>
       </c>
       <c r="F45" s="21">
         <f>ABS(MOD(C45-PT_mai+180,360)-180)</f>
@@ -1789,490 +1786,520 @@
         <v/>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="8" t="inlineStr">
+    <row r="46">
+      <c r="A46" s="12" t="inlineStr">
+        <is>
+          <t>Tây Bắc</t>
+        </is>
+      </c>
+      <c r="B46" s="14" t="inlineStr">
+        <is>
+          <t>NW</t>
+        </is>
+      </c>
+      <c r="C46" s="19" t="n">
+        <v>315</v>
+      </c>
+      <c r="D46" s="20" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="E46" s="20" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="F46" s="21">
+        <f>ABS(MOD(C46-PT_mai+180,360)-180)</f>
+        <v/>
+      </c>
+      <c r="G46" s="14">
+        <f>IF(F46&lt;=60,"Có – tính","Không")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
         <is>
           <t>F. BẢNG TRA (TCVN 8421:2010) – đồ thị đã đọc thành bảng, nội suy tuyến tính, ngoài bảng lấy giá trị biên</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="22" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="22" t="inlineStr">
         <is>
           <t>Hệ số kl quy đổi gió về mặt nước, địa hình dạng A (Bảng A3)</t>
         </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="23" t="inlineStr">
-        <is>
-          <t>Vl (m/s)</t>
-        </is>
-      </c>
-      <c r="B50" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="C50" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="D50" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="E50" s="24" t="n">
-        <v>25</v>
-      </c>
-      <c r="F50" s="24" t="n">
-        <v>30</v>
-      </c>
-      <c r="G50" s="24" t="n">
-        <v>35</v>
-      </c>
-      <c r="H50" s="24" t="n">
-        <v>40</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="23" t="inlineStr">
         <is>
+          <t>Vl (m/s)</t>
+        </is>
+      </c>
+      <c r="B51" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="C51" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="D51" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="E51" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="F51" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="G51" s="24" t="n">
+        <v>35</v>
+      </c>
+      <c r="H51" s="24" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="23" t="inlineStr">
+        <is>
           <t>kl</t>
         </is>
       </c>
-      <c r="B51" s="25" t="n">
+      <c r="B52" s="25" t="n">
         <v>1.1</v>
       </c>
-      <c r="C51" s="25" t="n">
+      <c r="C52" s="25" t="n">
         <v>1.1</v>
       </c>
-      <c r="D51" s="25" t="n">
+      <c r="D52" s="25" t="n">
         <v>1.09</v>
       </c>
-      <c r="E51" s="25" t="n">
+      <c r="E52" s="25" t="n">
         <v>1.09</v>
       </c>
-      <c r="F51" s="25" t="n">
+      <c r="F52" s="25" t="n">
         <v>1.09</v>
       </c>
-      <c r="G51" s="25" t="n">
+      <c r="G52" s="25" t="n">
         <v>1.09</v>
       </c>
-      <c r="H51" s="25" t="n">
+      <c r="H52" s="25" t="n">
         <v>1.08</v>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="22" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="22" t="inlineStr">
         <is>
           <t>Hệ số kα theo góc tới α (Bảng 9)</t>
         </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" s="23" t="inlineStr">
-        <is>
-          <t>α (°)</t>
-        </is>
-      </c>
-      <c r="B54" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="C54" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="D54" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="E54" s="24" t="n">
-        <v>30</v>
-      </c>
-      <c r="F54" s="24" t="n">
-        <v>40</v>
-      </c>
-      <c r="G54" s="24" t="n">
-        <v>50</v>
-      </c>
-      <c r="H54" s="24" t="n">
-        <v>60</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="23" t="inlineStr">
         <is>
+          <t>α (°)</t>
+        </is>
+      </c>
+      <c r="B55" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C55" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="D55" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="E55" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="F55" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="G55" s="24" t="n">
+        <v>50</v>
+      </c>
+      <c r="H55" s="24" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="23" t="inlineStr">
+        <is>
           <t>kα</t>
         </is>
       </c>
-      <c r="B55" s="25" t="n">
+      <c r="B56" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C55" s="25" t="n">
+      <c r="C56" s="25" t="n">
         <v>0.98</v>
       </c>
-      <c r="D55" s="25" t="n">
+      <c r="D56" s="25" t="n">
         <v>0.96</v>
       </c>
-      <c r="E55" s="25" t="n">
+      <c r="E56" s="25" t="n">
         <v>0.92</v>
       </c>
-      <c r="F55" s="25" t="n">
+      <c r="F56" s="25" t="n">
         <v>0.87</v>
       </c>
-      <c r="G55" s="25" t="n">
+      <c r="G56" s="25" t="n">
         <v>0.82</v>
       </c>
-      <c r="H55" s="25" t="n">
+      <c r="H56" s="25" t="n">
         <v>0.76</v>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="22" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="22" t="inlineStr">
         <is>
           <t>Hệ số nhám kr theo Δ/h1% (bảng hệ số nhám, thấm)</t>
         </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="23" t="inlineStr">
-        <is>
-          <t>Δ/h1%</t>
-        </is>
-      </c>
-      <c r="B58" s="26" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="C58" s="26" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="D58" s="26" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E58" s="26" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F58" s="26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G58" s="26" t="n">
-        <v>0.2</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="23" t="inlineStr">
         <is>
+          <t>Δ/h1%</t>
+        </is>
+      </c>
+      <c r="B59" s="26" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="C59" s="26" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D59" s="26" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E59" s="26" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F59" s="26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G59" s="26" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="23" t="inlineStr">
+        <is>
           <t>kr</t>
         </is>
       </c>
-      <c r="B59" s="25" t="n">
+      <c r="B60" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C59" s="25" t="n">
+      <c r="C60" s="25" t="n">
         <v>0.95</v>
       </c>
-      <c r="D59" s="25" t="n">
+      <c r="D60" s="25" t="n">
         <v>0.9</v>
       </c>
-      <c r="E59" s="25" t="n">
+      <c r="E60" s="25" t="n">
         <v>0.8</v>
       </c>
-      <c r="F59" s="25" t="n">
+      <c r="F60" s="25" t="n">
         <v>0.75</v>
       </c>
-      <c r="G59" s="25" t="n">
+      <c r="G60" s="25" t="n">
         <v>0.7</v>
       </c>
     </row>
-    <row r="61">
-      <c r="A61" s="22" t="inlineStr">
+    <row r="62">
+      <c r="A62" s="22" t="inlineStr">
         <is>
           <t>Hệ số thấm kp theo Δ/h1% (cùng bảng)</t>
         </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="23" t="inlineStr">
-        <is>
-          <t>Δ/h1%</t>
-        </is>
-      </c>
-      <c r="B62" s="26" t="n">
-        <v>0.002</v>
-      </c>
-      <c r="C62" s="26" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="D62" s="26" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E62" s="26" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="F62" s="26" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="G62" s="26" t="n">
-        <v>0.2</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="23" t="inlineStr">
         <is>
+          <t>Δ/h1%</t>
+        </is>
+      </c>
+      <c r="B63" s="26" t="n">
+        <v>0.002</v>
+      </c>
+      <c r="C63" s="26" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="D63" s="26" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="E63" s="26" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="F63" s="26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="G63" s="26" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="23" t="inlineStr">
+        <is>
           <t>kp</t>
         </is>
       </c>
-      <c r="B63" s="25" t="n">
+      <c r="B64" s="25" t="n">
         <v>0.9</v>
       </c>
-      <c r="C63" s="25" t="n">
+      <c r="C64" s="25" t="n">
         <v>0.85</v>
       </c>
-      <c r="D63" s="25" t="n">
+      <c r="D64" s="25" t="n">
         <v>0.8</v>
       </c>
-      <c r="E63" s="25" t="n">
+      <c r="E64" s="25" t="n">
         <v>0.7</v>
       </c>
-      <c r="F63" s="25" t="n">
+      <c r="F64" s="25" t="n">
         <v>0.6</v>
       </c>
-      <c r="G63" s="25" t="n">
+      <c r="G64" s="25" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="65">
-      <c r="A65" s="22" t="inlineStr">
+    <row r="66">
+      <c r="A66" s="22" t="inlineStr">
         <is>
           <t>Hệ số ksp theo V, hàng mái m = 3 ÷ 5 (m &lt; 3: 1,1 / 1,1 / 1,4; m &gt; 5: 0,6 / 1,2 / 1,6)</t>
         </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="23" t="inlineStr">
-        <is>
-          <t>V (m/s)</t>
-        </is>
-      </c>
-      <c r="B66" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="C66" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="D66" s="24" t="n">
-        <v>20</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="23" t="inlineStr">
         <is>
+          <t>V (m/s)</t>
+        </is>
+      </c>
+      <c r="B67" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C67" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="D67" s="24" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="23" t="inlineStr">
+        <is>
           <t>ksp</t>
         </is>
       </c>
-      <c r="B67" s="25" t="n">
+      <c r="B68" s="25" t="n">
         <v>0.8</v>
       </c>
-      <c r="C67" s="25" t="n">
+      <c r="C68" s="25" t="n">
         <v>1.1</v>
       </c>
-      <c r="D67" s="25" t="n">
+      <c r="D68" s="25" t="n">
         <v>1.5</v>
       </c>
     </row>
-    <row r="69">
-      <c r="A69" s="22" t="inlineStr">
+    <row r="70">
+      <c r="A70" s="22" t="inlineStr">
         <is>
           <t>Hệ số K1% theo gD/V² (đồ thị Hình 2)</t>
         </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="23" t="inlineStr">
-        <is>
-          <t>gD/V²</t>
-        </is>
-      </c>
-      <c r="B70" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="C70" s="24" t="n">
-        <v>100</v>
-      </c>
-      <c r="D70" s="24" t="n">
-        <v>153</v>
-      </c>
-      <c r="E70" s="24" t="n">
-        <v>514</v>
-      </c>
-      <c r="F70" s="24" t="n">
-        <v>1000</v>
-      </c>
-      <c r="G70" s="24" t="n">
-        <v>5000</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="23" t="inlineStr">
         <is>
-          <t>K1%</t>
-        </is>
-      </c>
-      <c r="B71" s="25" t="n">
-        <v>2</v>
-      </c>
-      <c r="C71" s="25" t="n">
-        <v>2.08</v>
-      </c>
-      <c r="D71" s="25" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="E71" s="25" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="F71" s="25" t="n">
-        <v>2.15</v>
-      </c>
-      <c r="G71" s="25" t="n">
-        <v>2.18</v>
+          <t>gD/V²</t>
+        </is>
+      </c>
+      <c r="B71" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="C71" s="24" t="n">
+        <v>100</v>
+      </c>
+      <c r="D71" s="24" t="n">
+        <v>153</v>
+      </c>
+      <c r="E71" s="24" t="n">
+        <v>514</v>
+      </c>
+      <c r="F71" s="24" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G71" s="24" t="n">
+        <v>5000</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="23" t="inlineStr">
         <is>
+          <t>K1%</t>
+        </is>
+      </c>
+      <c r="B72" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="C72" s="25" t="n">
+        <v>2.08</v>
+      </c>
+      <c r="D72" s="25" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="E72" s="25" t="n">
+        <v>2.13</v>
+      </c>
+      <c r="F72" s="25" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="G72" s="25" t="n">
+        <v>2.18</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="23" t="inlineStr">
+        <is>
           <t>lg(gD/V²)</t>
         </is>
       </c>
-      <c r="B72" s="27">
-        <f>LOG10(B70)</f>
-        <v/>
-      </c>
-      <c r="C72" s="27">
-        <f>LOG10(C70)</f>
-        <v/>
-      </c>
-      <c r="D72" s="27">
-        <f>LOG10(D70)</f>
-        <v/>
-      </c>
-      <c r="E72" s="27">
-        <f>LOG10(E70)</f>
-        <v/>
-      </c>
-      <c r="F72" s="27">
-        <f>LOG10(F70)</f>
-        <v/>
-      </c>
-      <c r="G72" s="27">
-        <f>LOG10(G70)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="22" t="inlineStr">
+      <c r="B73" s="27">
+        <f>LOG10(B71)</f>
+        <v/>
+      </c>
+      <c r="C73" s="27">
+        <f>LOG10(C71)</f>
+        <v/>
+      </c>
+      <c r="D73" s="27">
+        <f>LOG10(D71)</f>
+        <v/>
+      </c>
+      <c r="E73" s="27">
+        <f>LOG10(E71)</f>
+        <v/>
+      </c>
+      <c r="F73" s="27">
+        <f>LOG10(F71)</f>
+        <v/>
+      </c>
+      <c r="G73" s="27">
+        <f>LOG10(G71)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="22" t="inlineStr">
         <is>
           <t>Hệ số krun theo λ̄/h1%, mái m = 3 (đồ thị Hình 10)</t>
         </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="23" t="inlineStr">
-        <is>
-          <t>λ̄/h1%</t>
-        </is>
-      </c>
-      <c r="B75" s="24" t="n">
-        <v>5</v>
-      </c>
-      <c r="C75" s="24" t="n">
-        <v>8</v>
-      </c>
-      <c r="D75" s="24" t="n">
-        <v>10</v>
-      </c>
-      <c r="E75" s="24" t="n">
-        <v>12</v>
-      </c>
-      <c r="F75" s="24" t="n">
-        <v>15</v>
-      </c>
-      <c r="G75" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="H75" s="24" t="n">
-        <v>25</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="23" t="inlineStr">
         <is>
+          <t>λ̄/h1%</t>
+        </is>
+      </c>
+      <c r="B76" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C76" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="D76" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="E76" s="24" t="n">
+        <v>12</v>
+      </c>
+      <c r="F76" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="G76" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="H76" s="24" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="23" t="inlineStr">
+        <is>
           <t>krun</t>
         </is>
       </c>
-      <c r="B76" s="25" t="n">
+      <c r="B77" s="25" t="n">
         <v>1.2</v>
       </c>
-      <c r="C76" s="25" t="n">
+      <c r="C77" s="25" t="n">
         <v>1.4</v>
       </c>
-      <c r="D76" s="25" t="n">
+      <c r="D77" s="25" t="n">
         <v>1.48</v>
       </c>
-      <c r="E76" s="25" t="n">
+      <c r="E77" s="25" t="n">
         <v>1.57</v>
       </c>
-      <c r="F76" s="25" t="n">
+      <c r="F77" s="25" t="n">
         <v>1.7</v>
       </c>
-      <c r="G76" s="25" t="n">
+      <c r="G77" s="25" t="n">
         <v>1.84</v>
       </c>
-      <c r="H76" s="25" t="n">
+      <c r="H77" s="25" t="n">
         <v>1.95</v>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="22" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="22" t="inlineStr">
         <is>
           <t>Hệ số kw tính độ dềnh do gió (Bảng A2; V ≤ 20 m/s lấy 2,1·10⁻⁶ – bảng không có giá trị nhỏ hơn)</t>
         </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="23" t="inlineStr">
-        <is>
-          <t>V (m/s)</t>
-        </is>
-      </c>
-      <c r="B79" s="24" t="n">
-        <v>20</v>
-      </c>
-      <c r="C79" s="24" t="n">
-        <v>30</v>
-      </c>
-      <c r="D79" s="24" t="n">
-        <v>40</v>
-      </c>
-      <c r="E79" s="24" t="n">
-        <v>50</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="23" t="inlineStr">
         <is>
+          <t>V (m/s)</t>
+        </is>
+      </c>
+      <c r="B80" s="24" t="n">
+        <v>20</v>
+      </c>
+      <c r="C80" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="D80" s="24" t="n">
+        <v>40</v>
+      </c>
+      <c r="E80" s="24" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="23" t="inlineStr">
+        <is>
           <t>kw</t>
         </is>
       </c>
-      <c r="B80" s="28" t="n">
+      <c r="B81" s="28" t="n">
         <v>2.1e-06</v>
       </c>
-      <c r="C80" s="28" t="n">
+      <c r="C81" s="28" t="n">
         <v>3e-06</v>
       </c>
-      <c r="D80" s="28" t="n">
+      <c r="D81" s="28" t="n">
         <v>3.9e-06</v>
       </c>
-      <c r="E80" s="28" t="n">
+      <c r="E81" s="28" t="n">
         <v>4.8e-06</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="24">
+  <mergeCells count="25">
+    <mergeCell ref="D27:I27"/>
     <mergeCell ref="D13:I13"/>
     <mergeCell ref="D32:I32"/>
     <mergeCell ref="D16:I16"/>
@@ -2285,9 +2312,9 @@
     <mergeCell ref="D33:I33"/>
     <mergeCell ref="D24:I24"/>
     <mergeCell ref="D14:I14"/>
-    <mergeCell ref="D29:I29"/>
     <mergeCell ref="D5:I5"/>
     <mergeCell ref="D23:I23"/>
+    <mergeCell ref="D35:I35"/>
     <mergeCell ref="D20:I20"/>
     <mergeCell ref="D26:I26"/>
     <mergeCell ref="D19:I19"/>
@@ -2311,7 +2338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -3057,414 +3084,414 @@
     <row r="22">
       <c r="A22" s="29" t="inlineStr">
         <is>
-          <t>Hệ số K1%</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="inlineStr"/>
-      <c r="C22" s="34">
-        <f>IF(LOG10(C13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(C13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1))+(LOG10(C13)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))))</f>
-        <v/>
-      </c>
-      <c r="D22" s="34">
-        <f>IF(LOG10(D13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(D13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1))+(LOG10(D13)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))))</f>
-        <v/>
-      </c>
-      <c r="E22" s="34">
-        <f>IF(LOG10(E13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(E13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1))+(LOG10(E13)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))))</f>
-        <v/>
-      </c>
-      <c r="F22" s="34">
-        <f>IF(LOG10(F13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(F13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1))+(LOG10(F13)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))))</f>
-        <v/>
-      </c>
-      <c r="G22" s="34">
-        <f>IF(LOG10(G13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(G13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1))+(LOG10(G13)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))))</f>
-        <v/>
-      </c>
-      <c r="H22" s="34">
-        <f>IF(LOG10(H13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(H13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1))+(LOG10(H13)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))))</f>
+          <t>Độ sâu cơ thượng lưu dưới mực nước</t>
+        </is>
+      </c>
+      <c r="B22" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C22" s="32">
+        <f>C6-Z_co_TL</f>
+        <v/>
+      </c>
+      <c r="D22" s="32">
+        <f>D6-Z_co_TL</f>
+        <v/>
+      </c>
+      <c r="E22" s="32">
+        <f>E6-Z_co_TL</f>
+        <v/>
+      </c>
+      <c r="F22" s="32">
+        <f>F6-Z_co_TL</f>
+        <v/>
+      </c>
+      <c r="G22" s="32">
+        <f>G6-Z_co_TL</f>
+        <v/>
+      </c>
+      <c r="H22" s="32">
+        <f>H6-Z_co_TL</f>
         <v/>
       </c>
       <c r="I22" s="31" t="inlineStr">
         <is>
-          <t>Hình 2, theo gD/V²</t>
+          <t>Cơ thượng lưu +68,0 m</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="29" t="inlineStr">
         <is>
-          <t>Chiều cao sóng h1% = K1%·h̄</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C23" s="34">
-        <f>C22*C18</f>
-        <v/>
-      </c>
-      <c r="D23" s="34">
-        <f>D22*D18</f>
-        <v/>
-      </c>
-      <c r="E23" s="34">
-        <f>E22*E18</f>
-        <v/>
-      </c>
-      <c r="F23" s="34">
-        <f>F22*F18</f>
-        <v/>
-      </c>
-      <c r="G23" s="34">
-        <f>G22*G18</f>
-        <v/>
-      </c>
-      <c r="H23" s="34">
-        <f>H22*H18</f>
-        <v/>
-      </c>
-      <c r="I23" s="31" t="inlineStr"/>
+          <t>Kiểm tra cơ sâu hơn 0,5λ̄ (sóng chỉ leo trên đoạn mái m = 3,0)</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr"/>
+      <c r="C23" s="14">
+        <f>IF(C22&gt;0.5*C20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="D23" s="14">
+        <f>IF(D22&gt;0.5*D20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="E23" s="14">
+        <f>IF(E22&gt;0.5*E20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="F23" s="14">
+        <f>IF(F22&gt;0.5*F20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="G23" s="14">
+        <f>IF(G22&gt;0.5*G20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="H23" s="14">
+        <f>IF(H22&gt;0.5*H20,"Đúng","Xem lại")</f>
+        <v/>
+      </c>
+      <c r="I23" s="31" t="inlineStr">
+        <is>
+          <t>Đoạn mái m = 3,5 dưới cơ không ảnh hưởng sóng leo</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="29" t="inlineStr">
         <is>
-          <t>Độ nhám tương đối Δ/h1%</t>
+          <t>Hệ số K1%</t>
         </is>
       </c>
       <c r="B24" s="14" t="inlineStr"/>
-      <c r="C24" s="35">
-        <f>Delta_n/C23</f>
-        <v/>
-      </c>
-      <c r="D24" s="35">
-        <f>Delta_n/D23</f>
-        <v/>
-      </c>
-      <c r="E24" s="35">
-        <f>Delta_n/E23</f>
-        <v/>
-      </c>
-      <c r="F24" s="35">
-        <f>Delta_n/F23</f>
-        <v/>
-      </c>
-      <c r="G24" s="35">
-        <f>Delta_n/G23</f>
-        <v/>
-      </c>
-      <c r="H24" s="35">
-        <f>Delta_n/H23</f>
+      <c r="C24" s="34">
+        <f>IF(LOG10(C13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(C13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1))+(LOG10(C13)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(C13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(C13),K1_lg,1)))))</f>
+        <v/>
+      </c>
+      <c r="D24" s="34">
+        <f>IF(LOG10(D13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(D13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1))+(LOG10(D13)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(D13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(D13),K1_lg,1)))))</f>
+        <v/>
+      </c>
+      <c r="E24" s="34">
+        <f>IF(LOG10(E13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(E13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1))+(LOG10(E13)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(E13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(E13),K1_lg,1)))))</f>
+        <v/>
+      </c>
+      <c r="F24" s="34">
+        <f>IF(LOG10(F13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(F13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1))+(LOG10(F13)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(F13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(F13),K1_lg,1)))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="34">
+        <f>IF(LOG10(G13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(G13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1))+(LOG10(G13)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(G13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(G13),K1_lg,1)))))</f>
+        <v/>
+      </c>
+      <c r="H24" s="34">
+        <f>IF(LOG10(H13)&lt;=INDEX(K1_lg,1),INDEX(K1_k,1),IF(LOG10(H13)&gt;=INDEX(K1_lg,COUNT(K1_lg)),INDEX(K1_k,COUNT(K1_lg)),INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1))+(LOG10(H13)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))*(INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_k,MATCH(LOG10(H13),K1_lg,1)))/(INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)+1)-INDEX(K1_lg,MATCH(LOG10(H13),K1_lg,1)))))</f>
         <v/>
       </c>
       <c r="I24" s="31" t="inlineStr">
         <is>
-          <t>Δ = 0,02 m</t>
+          <t>Hình 2, theo gD/V²</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="29" t="inlineStr">
         <is>
-          <t>Hệ số nhám kr</t>
-        </is>
-      </c>
-      <c r="B25" s="14" t="inlineStr"/>
+          <t>Chiều cao sóng h1% = K1%·h̄</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
       <c r="C25" s="34">
-        <f>IF(C24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(C24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(C24,KR_x,1))+(C24-INDEX(KR_x,MATCH(C24,KR_x,1)))*(INDEX(KR_kr,MATCH(C24,KR_x,1)+1)-INDEX(KR_kr,MATCH(C24,KR_x,1)))/(INDEX(KR_x,MATCH(C24,KR_x,1)+1)-INDEX(KR_x,MATCH(C24,KR_x,1)))))</f>
+        <f>C24*C18</f>
         <v/>
       </c>
       <c r="D25" s="34">
-        <f>IF(D24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(D24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(D24,KR_x,1))+(D24-INDEX(KR_x,MATCH(D24,KR_x,1)))*(INDEX(KR_kr,MATCH(D24,KR_x,1)+1)-INDEX(KR_kr,MATCH(D24,KR_x,1)))/(INDEX(KR_x,MATCH(D24,KR_x,1)+1)-INDEX(KR_x,MATCH(D24,KR_x,1)))))</f>
+        <f>D24*D18</f>
         <v/>
       </c>
       <c r="E25" s="34">
-        <f>IF(E24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(E24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(E24,KR_x,1))+(E24-INDEX(KR_x,MATCH(E24,KR_x,1)))*(INDEX(KR_kr,MATCH(E24,KR_x,1)+1)-INDEX(KR_kr,MATCH(E24,KR_x,1)))/(INDEX(KR_x,MATCH(E24,KR_x,1)+1)-INDEX(KR_x,MATCH(E24,KR_x,1)))))</f>
+        <f>E24*E18</f>
         <v/>
       </c>
       <c r="F25" s="34">
-        <f>IF(F24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(F24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(F24,KR_x,1))+(F24-INDEX(KR_x,MATCH(F24,KR_x,1)))*(INDEX(KR_kr,MATCH(F24,KR_x,1)+1)-INDEX(KR_kr,MATCH(F24,KR_x,1)))/(INDEX(KR_x,MATCH(F24,KR_x,1)+1)-INDEX(KR_x,MATCH(F24,KR_x,1)))))</f>
+        <f>F24*F18</f>
         <v/>
       </c>
       <c r="G25" s="34">
-        <f>IF(G24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(G24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(G24,KR_x,1))+(G24-INDEX(KR_x,MATCH(G24,KR_x,1)))*(INDEX(KR_kr,MATCH(G24,KR_x,1)+1)-INDEX(KR_kr,MATCH(G24,KR_x,1)))/(INDEX(KR_x,MATCH(G24,KR_x,1)+1)-INDEX(KR_x,MATCH(G24,KR_x,1)))))</f>
+        <f>G24*G18</f>
         <v/>
       </c>
       <c r="H25" s="34">
-        <f>IF(H24&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(H24&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(H24,KR_x,1))+(H24-INDEX(KR_x,MATCH(H24,KR_x,1)))*(INDEX(KR_kr,MATCH(H24,KR_x,1)+1)-INDEX(KR_kr,MATCH(H24,KR_x,1)))/(INDEX(KR_x,MATCH(H24,KR_x,1)+1)-INDEX(KR_x,MATCH(H24,KR_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="I25" s="31" t="inlineStr">
-        <is>
-          <t>Bảng hệ số nhám, thấm</t>
-        </is>
-      </c>
+        <f>H24*H18</f>
+        <v/>
+      </c>
+      <c r="I25" s="31" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="29" t="inlineStr">
         <is>
-          <t>Hệ số thấm kp</t>
+          <t>Độ nhám tương đối Δ/h1%</t>
         </is>
       </c>
       <c r="B26" s="14" t="inlineStr"/>
-      <c r="C26" s="34">
-        <f>IF(C24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(C24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(C24,KP_x,1))+(C24-INDEX(KP_x,MATCH(C24,KP_x,1)))*(INDEX(KP_kp,MATCH(C24,KP_x,1)+1)-INDEX(KP_kp,MATCH(C24,KP_x,1)))/(INDEX(KP_x,MATCH(C24,KP_x,1)+1)-INDEX(KP_x,MATCH(C24,KP_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="D26" s="34">
-        <f>IF(D24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(D24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(D24,KP_x,1))+(D24-INDEX(KP_x,MATCH(D24,KP_x,1)))*(INDEX(KP_kp,MATCH(D24,KP_x,1)+1)-INDEX(KP_kp,MATCH(D24,KP_x,1)))/(INDEX(KP_x,MATCH(D24,KP_x,1)+1)-INDEX(KP_x,MATCH(D24,KP_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="E26" s="34">
-        <f>IF(E24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(E24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(E24,KP_x,1))+(E24-INDEX(KP_x,MATCH(E24,KP_x,1)))*(INDEX(KP_kp,MATCH(E24,KP_x,1)+1)-INDEX(KP_kp,MATCH(E24,KP_x,1)))/(INDEX(KP_x,MATCH(E24,KP_x,1)+1)-INDEX(KP_x,MATCH(E24,KP_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="F26" s="34">
-        <f>IF(F24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(F24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(F24,KP_x,1))+(F24-INDEX(KP_x,MATCH(F24,KP_x,1)))*(INDEX(KP_kp,MATCH(F24,KP_x,1)+1)-INDEX(KP_kp,MATCH(F24,KP_x,1)))/(INDEX(KP_x,MATCH(F24,KP_x,1)+1)-INDEX(KP_x,MATCH(F24,KP_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="G26" s="34">
-        <f>IF(G24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(G24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(G24,KP_x,1))+(G24-INDEX(KP_x,MATCH(G24,KP_x,1)))*(INDEX(KP_kp,MATCH(G24,KP_x,1)+1)-INDEX(KP_kp,MATCH(G24,KP_x,1)))/(INDEX(KP_x,MATCH(G24,KP_x,1)+1)-INDEX(KP_x,MATCH(G24,KP_x,1)))))</f>
-        <v/>
-      </c>
-      <c r="H26" s="34">
-        <f>IF(H24&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(H24&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(H24,KP_x,1))+(H24-INDEX(KP_x,MATCH(H24,KP_x,1)))*(INDEX(KP_kp,MATCH(H24,KP_x,1)+1)-INDEX(KP_kp,MATCH(H24,KP_x,1)))/(INDEX(KP_x,MATCH(H24,KP_x,1)+1)-INDEX(KP_x,MATCH(H24,KP_x,1)))))</f>
+      <c r="C26" s="35">
+        <f>Delta_n/C25</f>
+        <v/>
+      </c>
+      <c r="D26" s="35">
+        <f>Delta_n/D25</f>
+        <v/>
+      </c>
+      <c r="E26" s="35">
+        <f>Delta_n/E25</f>
+        <v/>
+      </c>
+      <c r="F26" s="35">
+        <f>Delta_n/F25</f>
+        <v/>
+      </c>
+      <c r="G26" s="35">
+        <f>Delta_n/G25</f>
+        <v/>
+      </c>
+      <c r="H26" s="35">
+        <f>Delta_n/H25</f>
         <v/>
       </c>
       <c r="I26" s="31" t="inlineStr">
         <is>
-          <t>Như trên</t>
+          <t>Δ = 0,02 m</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="29" t="inlineStr">
         <is>
-          <t>Hệ số ksp</t>
+          <t>Hệ số nhám kr</t>
         </is>
       </c>
       <c r="B27" s="14" t="inlineStr"/>
       <c r="C27" s="34">
-        <f>IF(C10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(C10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(C10,KSP_V,1))+(C10-INDEX(KSP_V,MATCH(C10,KSP_V,1)))*(INDEX(KSP_k,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(C10,KSP_V,1)))/(INDEX(KSP_V,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(C10,KSP_V,1)))))</f>
+        <f>IF(C26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(C26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(C26,KR_x,1))+(C26-INDEX(KR_x,MATCH(C26,KR_x,1)))*(INDEX(KR_kr,MATCH(C26,KR_x,1)+1)-INDEX(KR_kr,MATCH(C26,KR_x,1)))/(INDEX(KR_x,MATCH(C26,KR_x,1)+1)-INDEX(KR_x,MATCH(C26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="D27" s="34">
-        <f>IF(D10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(D10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(D10,KSP_V,1))+(D10-INDEX(KSP_V,MATCH(D10,KSP_V,1)))*(INDEX(KSP_k,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(D10,KSP_V,1)))/(INDEX(KSP_V,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(D10,KSP_V,1)))))</f>
+        <f>IF(D26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(D26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(D26,KR_x,1))+(D26-INDEX(KR_x,MATCH(D26,KR_x,1)))*(INDEX(KR_kr,MATCH(D26,KR_x,1)+1)-INDEX(KR_kr,MATCH(D26,KR_x,1)))/(INDEX(KR_x,MATCH(D26,KR_x,1)+1)-INDEX(KR_x,MATCH(D26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="E27" s="34">
-        <f>IF(E10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(E10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(E10,KSP_V,1))+(E10-INDEX(KSP_V,MATCH(E10,KSP_V,1)))*(INDEX(KSP_k,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(E10,KSP_V,1)))/(INDEX(KSP_V,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(E10,KSP_V,1)))))</f>
+        <f>IF(E26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(E26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(E26,KR_x,1))+(E26-INDEX(KR_x,MATCH(E26,KR_x,1)))*(INDEX(KR_kr,MATCH(E26,KR_x,1)+1)-INDEX(KR_kr,MATCH(E26,KR_x,1)))/(INDEX(KR_x,MATCH(E26,KR_x,1)+1)-INDEX(KR_x,MATCH(E26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="F27" s="34">
-        <f>IF(F10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(F10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(F10,KSP_V,1))+(F10-INDEX(KSP_V,MATCH(F10,KSP_V,1)))*(INDEX(KSP_k,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(F10,KSP_V,1)))/(INDEX(KSP_V,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(F10,KSP_V,1)))))</f>
+        <f>IF(F26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(F26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(F26,KR_x,1))+(F26-INDEX(KR_x,MATCH(F26,KR_x,1)))*(INDEX(KR_kr,MATCH(F26,KR_x,1)+1)-INDEX(KR_kr,MATCH(F26,KR_x,1)))/(INDEX(KR_x,MATCH(F26,KR_x,1)+1)-INDEX(KR_x,MATCH(F26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="G27" s="34">
-        <f>IF(G10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(G10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(G10,KSP_V,1))+(G10-INDEX(KSP_V,MATCH(G10,KSP_V,1)))*(INDEX(KSP_k,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(G10,KSP_V,1)))/(INDEX(KSP_V,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(G10,KSP_V,1)))))</f>
+        <f>IF(G26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(G26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(G26,KR_x,1))+(G26-INDEX(KR_x,MATCH(G26,KR_x,1)))*(INDEX(KR_kr,MATCH(G26,KR_x,1)+1)-INDEX(KR_kr,MATCH(G26,KR_x,1)))/(INDEX(KR_x,MATCH(G26,KR_x,1)+1)-INDEX(KR_x,MATCH(G26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="H27" s="34">
-        <f>IF(H10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(H10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(H10,KSP_V,1))+(H10-INDEX(KSP_V,MATCH(H10,KSP_V,1)))*(INDEX(KSP_k,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(H10,KSP_V,1)))/(INDEX(KSP_V,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(H10,KSP_V,1)))))</f>
+        <f>IF(H26&lt;=INDEX(KR_x,1),INDEX(KR_kr,1),IF(H26&gt;=INDEX(KR_x,COUNT(KR_x)),INDEX(KR_kr,COUNT(KR_x)),INDEX(KR_kr,MATCH(H26,KR_x,1))+(H26-INDEX(KR_x,MATCH(H26,KR_x,1)))*(INDEX(KR_kr,MATCH(H26,KR_x,1)+1)-INDEX(KR_kr,MATCH(H26,KR_x,1)))/(INDEX(KR_x,MATCH(H26,KR_x,1)+1)-INDEX(KR_x,MATCH(H26,KR_x,1)))))</f>
         <v/>
       </c>
       <c r="I27" s="31" t="inlineStr">
         <is>
-          <t>Bảng ksp, mái m = 3 ÷ 5</t>
+          <t>Bảng hệ số nhám, thấm</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="29" t="inlineStr">
         <is>
-          <t>Độ thoải sóng λ̄/h1%</t>
+          <t>Hệ số thấm kp</t>
         </is>
       </c>
       <c r="B28" s="14" t="inlineStr"/>
-      <c r="C28" s="32">
-        <f>C20/C23</f>
-        <v/>
-      </c>
-      <c r="D28" s="32">
-        <f>D20/D23</f>
-        <v/>
-      </c>
-      <c r="E28" s="32">
-        <f>E20/E23</f>
-        <v/>
-      </c>
-      <c r="F28" s="32">
-        <f>F20/F23</f>
-        <v/>
-      </c>
-      <c r="G28" s="32">
-        <f>G20/G23</f>
-        <v/>
-      </c>
-      <c r="H28" s="32">
-        <f>H20/H23</f>
-        <v/>
-      </c>
-      <c r="I28" s="31" t="inlineStr"/>
+      <c r="C28" s="34">
+        <f>IF(C26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(C26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(C26,KP_x,1))+(C26-INDEX(KP_x,MATCH(C26,KP_x,1)))*(INDEX(KP_kp,MATCH(C26,KP_x,1)+1)-INDEX(KP_kp,MATCH(C26,KP_x,1)))/(INDEX(KP_x,MATCH(C26,KP_x,1)+1)-INDEX(KP_x,MATCH(C26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="D28" s="34">
+        <f>IF(D26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(D26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(D26,KP_x,1))+(D26-INDEX(KP_x,MATCH(D26,KP_x,1)))*(INDEX(KP_kp,MATCH(D26,KP_x,1)+1)-INDEX(KP_kp,MATCH(D26,KP_x,1)))/(INDEX(KP_x,MATCH(D26,KP_x,1)+1)-INDEX(KP_x,MATCH(D26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="E28" s="34">
+        <f>IF(E26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(E26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(E26,KP_x,1))+(E26-INDEX(KP_x,MATCH(E26,KP_x,1)))*(INDEX(KP_kp,MATCH(E26,KP_x,1)+1)-INDEX(KP_kp,MATCH(E26,KP_x,1)))/(INDEX(KP_x,MATCH(E26,KP_x,1)+1)-INDEX(KP_x,MATCH(E26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="F28" s="34">
+        <f>IF(F26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(F26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(F26,KP_x,1))+(F26-INDEX(KP_x,MATCH(F26,KP_x,1)))*(INDEX(KP_kp,MATCH(F26,KP_x,1)+1)-INDEX(KP_kp,MATCH(F26,KP_x,1)))/(INDEX(KP_x,MATCH(F26,KP_x,1)+1)-INDEX(KP_x,MATCH(F26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="G28" s="34">
+        <f>IF(G26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(G26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(G26,KP_x,1))+(G26-INDEX(KP_x,MATCH(G26,KP_x,1)))*(INDEX(KP_kp,MATCH(G26,KP_x,1)+1)-INDEX(KP_kp,MATCH(G26,KP_x,1)))/(INDEX(KP_x,MATCH(G26,KP_x,1)+1)-INDEX(KP_x,MATCH(G26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="H28" s="34">
+        <f>IF(H26&lt;=INDEX(KP_x,1),INDEX(KP_kp,1),IF(H26&gt;=INDEX(KP_x,COUNT(KP_x)),INDEX(KP_kp,COUNT(KP_x)),INDEX(KP_kp,MATCH(H26,KP_x,1))+(H26-INDEX(KP_x,MATCH(H26,KP_x,1)))*(INDEX(KP_kp,MATCH(H26,KP_x,1)+1)-INDEX(KP_kp,MATCH(H26,KP_x,1)))/(INDEX(KP_x,MATCH(H26,KP_x,1)+1)-INDEX(KP_x,MATCH(H26,KP_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="I28" s="31" t="inlineStr">
+        <is>
+          <t>Như trên</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="29" t="inlineStr">
         <is>
-          <t>Hệ số krun</t>
+          <t>Hệ số ksp</t>
         </is>
       </c>
       <c r="B29" s="14" t="inlineStr"/>
       <c r="C29" s="34">
-        <f>IF(C28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(C28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(C28,KRUN_x,1))+(C28-INDEX(KRUN_x,MATCH(C28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(C28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(C28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(C28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(C28,KRUN_x,1)))))</f>
+        <f>IF(C10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(C10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(C10,KSP_V,1))+(C10-INDEX(KSP_V,MATCH(C10,KSP_V,1)))*(INDEX(KSP_k,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(C10,KSP_V,1)))/(INDEX(KSP_V,MATCH(C10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(C10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="D29" s="34">
-        <f>IF(D28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(D28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(D28,KRUN_x,1))+(D28-INDEX(KRUN_x,MATCH(D28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(D28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(D28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(D28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(D28,KRUN_x,1)))))</f>
+        <f>IF(D10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(D10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(D10,KSP_V,1))+(D10-INDEX(KSP_V,MATCH(D10,KSP_V,1)))*(INDEX(KSP_k,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(D10,KSP_V,1)))/(INDEX(KSP_V,MATCH(D10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(D10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="E29" s="34">
-        <f>IF(E28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(E28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(E28,KRUN_x,1))+(E28-INDEX(KRUN_x,MATCH(E28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(E28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(E28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(E28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(E28,KRUN_x,1)))))</f>
+        <f>IF(E10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(E10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(E10,KSP_V,1))+(E10-INDEX(KSP_V,MATCH(E10,KSP_V,1)))*(INDEX(KSP_k,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(E10,KSP_V,1)))/(INDEX(KSP_V,MATCH(E10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(E10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="F29" s="34">
-        <f>IF(F28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(F28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(F28,KRUN_x,1))+(F28-INDEX(KRUN_x,MATCH(F28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(F28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(F28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(F28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(F28,KRUN_x,1)))))</f>
+        <f>IF(F10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(F10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(F10,KSP_V,1))+(F10-INDEX(KSP_V,MATCH(F10,KSP_V,1)))*(INDEX(KSP_k,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(F10,KSP_V,1)))/(INDEX(KSP_V,MATCH(F10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(F10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="G29" s="34">
-        <f>IF(G28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(G28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(G28,KRUN_x,1))+(G28-INDEX(KRUN_x,MATCH(G28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(G28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(G28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(G28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(G28,KRUN_x,1)))))</f>
+        <f>IF(G10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(G10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(G10,KSP_V,1))+(G10-INDEX(KSP_V,MATCH(G10,KSP_V,1)))*(INDEX(KSP_k,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(G10,KSP_V,1)))/(INDEX(KSP_V,MATCH(G10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(G10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="H29" s="34">
-        <f>IF(H28&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(H28&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(H28,KRUN_x,1))+(H28-INDEX(KRUN_x,MATCH(H28,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(H28,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(H28,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(H28,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(H28,KRUN_x,1)))))</f>
+        <f>IF(H10&lt;=INDEX(KSP_V,1),INDEX(KSP_k,1),IF(H10&gt;=INDEX(KSP_V,COUNT(KSP_V)),INDEX(KSP_k,COUNT(KSP_V)),INDEX(KSP_k,MATCH(H10,KSP_V,1))+(H10-INDEX(KSP_V,MATCH(H10,KSP_V,1)))*(INDEX(KSP_k,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_k,MATCH(H10,KSP_V,1)))/(INDEX(KSP_V,MATCH(H10,KSP_V,1)+1)-INDEX(KSP_V,MATCH(H10,KSP_V,1)))))</f>
         <v/>
       </c>
       <c r="I29" s="31" t="inlineStr">
         <is>
-          <t>Hình 10, mái m = 3</t>
+          <t>Bảng ksp, mái m = 3 ÷ 5</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="29" t="inlineStr">
         <is>
-          <t>Hệ số kα</t>
+          <t>Độ thoải sóng λ̄/h1%</t>
         </is>
       </c>
       <c r="B30" s="14" t="inlineStr"/>
-      <c r="C30" s="34">
-        <f>IF(C11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(C11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(C11,KA_goc,1))+(C11-INDEX(KA_goc,MATCH(C11,KA_goc,1)))*(INDEX(KA_k,MATCH(C11,KA_goc,1)+1)-INDEX(KA_k,MATCH(C11,KA_goc,1)))/(INDEX(KA_goc,MATCH(C11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(C11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="D30" s="34">
-        <f>IF(D11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(D11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(D11,KA_goc,1))+(D11-INDEX(KA_goc,MATCH(D11,KA_goc,1)))*(INDEX(KA_k,MATCH(D11,KA_goc,1)+1)-INDEX(KA_k,MATCH(D11,KA_goc,1)))/(INDEX(KA_goc,MATCH(D11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(D11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="E30" s="34">
-        <f>IF(E11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(E11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(E11,KA_goc,1))+(E11-INDEX(KA_goc,MATCH(E11,KA_goc,1)))*(INDEX(KA_k,MATCH(E11,KA_goc,1)+1)-INDEX(KA_k,MATCH(E11,KA_goc,1)))/(INDEX(KA_goc,MATCH(E11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(E11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="F30" s="34">
-        <f>IF(F11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(F11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(F11,KA_goc,1))+(F11-INDEX(KA_goc,MATCH(F11,KA_goc,1)))*(INDEX(KA_k,MATCH(F11,KA_goc,1)+1)-INDEX(KA_k,MATCH(F11,KA_goc,1)))/(INDEX(KA_goc,MATCH(F11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(F11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="G30" s="34">
-        <f>IF(G11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(G11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(G11,KA_goc,1))+(G11-INDEX(KA_goc,MATCH(G11,KA_goc,1)))*(INDEX(KA_k,MATCH(G11,KA_goc,1)+1)-INDEX(KA_k,MATCH(G11,KA_goc,1)))/(INDEX(KA_goc,MATCH(G11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(G11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="H30" s="34">
-        <f>IF(H11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(H11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(H11,KA_goc,1))+(H11-INDEX(KA_goc,MATCH(H11,KA_goc,1)))*(INDEX(KA_k,MATCH(H11,KA_goc,1)+1)-INDEX(KA_k,MATCH(H11,KA_goc,1)))/(INDEX(KA_goc,MATCH(H11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(H11,KA_goc,1)))))</f>
-        <v/>
-      </c>
-      <c r="I30" s="31" t="inlineStr">
-        <is>
-          <t>Bảng 9, theo α</t>
-        </is>
-      </c>
+      <c r="C30" s="32">
+        <f>C20/C25</f>
+        <v/>
+      </c>
+      <c r="D30" s="32">
+        <f>D20/D25</f>
+        <v/>
+      </c>
+      <c r="E30" s="32">
+        <f>E20/E25</f>
+        <v/>
+      </c>
+      <c r="F30" s="32">
+        <f>F20/F25</f>
+        <v/>
+      </c>
+      <c r="G30" s="32">
+        <f>G20/G25</f>
+        <v/>
+      </c>
+      <c r="H30" s="32">
+        <f>H20/H25</f>
+        <v/>
+      </c>
+      <c r="I30" s="31" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="36" t="inlineStr">
-        <is>
-          <t>Chiều cao sóng leo hsl1%</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C31" s="27">
-        <f>C25*C26*C27*C29*C30*C23</f>
-        <v/>
-      </c>
-      <c r="D31" s="27">
-        <f>D25*D26*D27*D29*D30*D23</f>
-        <v/>
-      </c>
-      <c r="E31" s="27">
-        <f>E25*E26*E27*E29*E30*E23</f>
-        <v/>
-      </c>
-      <c r="F31" s="27">
-        <f>F25*F26*F27*F29*F30*F23</f>
-        <v/>
-      </c>
-      <c r="G31" s="27">
-        <f>G25*G26*G27*G29*G30*G23</f>
-        <v/>
-      </c>
-      <c r="H31" s="27">
-        <f>H25*H26*H27*H29*H30*H23</f>
+      <c r="A31" s="29" t="inlineStr">
+        <is>
+          <t>Hệ số krun</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="inlineStr"/>
+      <c r="C31" s="34">
+        <f>IF(C30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(C30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(C30,KRUN_x,1))+(C30-INDEX(KRUN_x,MATCH(C30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(C30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(C30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(C30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(C30,KRUN_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="D31" s="34">
+        <f>IF(D30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(D30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(D30,KRUN_x,1))+(D30-INDEX(KRUN_x,MATCH(D30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(D30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(D30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(D30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(D30,KRUN_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="E31" s="34">
+        <f>IF(E30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(E30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(E30,KRUN_x,1))+(E30-INDEX(KRUN_x,MATCH(E30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(E30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(E30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(E30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(E30,KRUN_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="F31" s="34">
+        <f>IF(F30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(F30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(F30,KRUN_x,1))+(F30-INDEX(KRUN_x,MATCH(F30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(F30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(F30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(F30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(F30,KRUN_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="G31" s="34">
+        <f>IF(G30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(G30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(G30,KRUN_x,1))+(G30-INDEX(KRUN_x,MATCH(G30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(G30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(G30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(G30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(G30,KRUN_x,1)))))</f>
+        <v/>
+      </c>
+      <c r="H31" s="34">
+        <f>IF(H30&lt;=INDEX(KRUN_x,1),INDEX(KRUN_k,1),IF(H30&gt;=INDEX(KRUN_x,COUNT(KRUN_x)),INDEX(KRUN_k,COUNT(KRUN_x)),INDEX(KRUN_k,MATCH(H30,KRUN_x,1))+(H30-INDEX(KRUN_x,MATCH(H30,KRUN_x,1)))*(INDEX(KRUN_k,MATCH(H30,KRUN_x,1)+1)-INDEX(KRUN_k,MATCH(H30,KRUN_x,1)))/(INDEX(KRUN_x,MATCH(H30,KRUN_x,1)+1)-INDEX(KRUN_x,MATCH(H30,KRUN_x,1)))))</f>
         <v/>
       </c>
       <c r="I31" s="31" t="inlineStr">
         <is>
-          <t>hsl1% = kr·kp·ksp·krun·kα·h1%</t>
+          <t>Hình 10, mái m = 3</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="29" t="inlineStr">
         <is>
-          <t>Hệ số kw</t>
+          <t>Hệ số kα</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr"/>
-      <c r="C32" s="37">
-        <f>IF(C10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(C10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(C10,KW_V,1))+(C10-INDEX(KW_V,MATCH(C10,KW_V,1)))*(INDEX(KW_k,MATCH(C10,KW_V,1)+1)-INDEX(KW_k,MATCH(C10,KW_V,1)))/(INDEX(KW_V,MATCH(C10,KW_V,1)+1)-INDEX(KW_V,MATCH(C10,KW_V,1)))))</f>
-        <v/>
-      </c>
-      <c r="D32" s="37">
-        <f>IF(D10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(D10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(D10,KW_V,1))+(D10-INDEX(KW_V,MATCH(D10,KW_V,1)))*(INDEX(KW_k,MATCH(D10,KW_V,1)+1)-INDEX(KW_k,MATCH(D10,KW_V,1)))/(INDEX(KW_V,MATCH(D10,KW_V,1)+1)-INDEX(KW_V,MATCH(D10,KW_V,1)))))</f>
-        <v/>
-      </c>
-      <c r="E32" s="37">
-        <f>IF(E10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(E10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(E10,KW_V,1))+(E10-INDEX(KW_V,MATCH(E10,KW_V,1)))*(INDEX(KW_k,MATCH(E10,KW_V,1)+1)-INDEX(KW_k,MATCH(E10,KW_V,1)))/(INDEX(KW_V,MATCH(E10,KW_V,1)+1)-INDEX(KW_V,MATCH(E10,KW_V,1)))))</f>
-        <v/>
-      </c>
-      <c r="F32" s="37">
-        <f>IF(F10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(F10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(F10,KW_V,1))+(F10-INDEX(KW_V,MATCH(F10,KW_V,1)))*(INDEX(KW_k,MATCH(F10,KW_V,1)+1)-INDEX(KW_k,MATCH(F10,KW_V,1)))/(INDEX(KW_V,MATCH(F10,KW_V,1)+1)-INDEX(KW_V,MATCH(F10,KW_V,1)))))</f>
-        <v/>
-      </c>
-      <c r="G32" s="37">
-        <f>IF(G10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(G10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(G10,KW_V,1))+(G10-INDEX(KW_V,MATCH(G10,KW_V,1)))*(INDEX(KW_k,MATCH(G10,KW_V,1)+1)-INDEX(KW_k,MATCH(G10,KW_V,1)))/(INDEX(KW_V,MATCH(G10,KW_V,1)+1)-INDEX(KW_V,MATCH(G10,KW_V,1)))))</f>
-        <v/>
-      </c>
-      <c r="H32" s="37">
-        <f>IF(H10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(H10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(H10,KW_V,1))+(H10-INDEX(KW_V,MATCH(H10,KW_V,1)))*(INDEX(KW_k,MATCH(H10,KW_V,1)+1)-INDEX(KW_k,MATCH(H10,KW_V,1)))/(INDEX(KW_V,MATCH(H10,KW_V,1)+1)-INDEX(KW_V,MATCH(H10,KW_V,1)))))</f>
+      <c r="C32" s="34">
+        <f>IF(C11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(C11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(C11,KA_goc,1))+(C11-INDEX(KA_goc,MATCH(C11,KA_goc,1)))*(INDEX(KA_k,MATCH(C11,KA_goc,1)+1)-INDEX(KA_k,MATCH(C11,KA_goc,1)))/(INDEX(KA_goc,MATCH(C11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(C11,KA_goc,1)))))</f>
+        <v/>
+      </c>
+      <c r="D32" s="34">
+        <f>IF(D11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(D11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(D11,KA_goc,1))+(D11-INDEX(KA_goc,MATCH(D11,KA_goc,1)))*(INDEX(KA_k,MATCH(D11,KA_goc,1)+1)-INDEX(KA_k,MATCH(D11,KA_goc,1)))/(INDEX(KA_goc,MATCH(D11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(D11,KA_goc,1)))))</f>
+        <v/>
+      </c>
+      <c r="E32" s="34">
+        <f>IF(E11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(E11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(E11,KA_goc,1))+(E11-INDEX(KA_goc,MATCH(E11,KA_goc,1)))*(INDEX(KA_k,MATCH(E11,KA_goc,1)+1)-INDEX(KA_k,MATCH(E11,KA_goc,1)))/(INDEX(KA_goc,MATCH(E11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(E11,KA_goc,1)))))</f>
+        <v/>
+      </c>
+      <c r="F32" s="34">
+        <f>IF(F11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(F11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(F11,KA_goc,1))+(F11-INDEX(KA_goc,MATCH(F11,KA_goc,1)))*(INDEX(KA_k,MATCH(F11,KA_goc,1)+1)-INDEX(KA_k,MATCH(F11,KA_goc,1)))/(INDEX(KA_goc,MATCH(F11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(F11,KA_goc,1)))))</f>
+        <v/>
+      </c>
+      <c r="G32" s="34">
+        <f>IF(G11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(G11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(G11,KA_goc,1))+(G11-INDEX(KA_goc,MATCH(G11,KA_goc,1)))*(INDEX(KA_k,MATCH(G11,KA_goc,1)+1)-INDEX(KA_k,MATCH(G11,KA_goc,1)))/(INDEX(KA_goc,MATCH(G11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(G11,KA_goc,1)))))</f>
+        <v/>
+      </c>
+      <c r="H32" s="34">
+        <f>IF(H11&lt;=INDEX(KA_goc,1),INDEX(KA_k,1),IF(H11&gt;=INDEX(KA_goc,COUNT(KA_goc)),INDEX(KA_k,COUNT(KA_goc)),INDEX(KA_k,MATCH(H11,KA_goc,1))+(H11-INDEX(KA_goc,MATCH(H11,KA_goc,1)))*(INDEX(KA_k,MATCH(H11,KA_goc,1)+1)-INDEX(KA_k,MATCH(H11,KA_goc,1)))/(INDEX(KA_goc,MATCH(H11,KA_goc,1)+1)-INDEX(KA_goc,MATCH(H11,KA_goc,1)))))</f>
         <v/>
       </c>
       <c r="I32" s="31" t="inlineStr">
         <is>
-          <t>Bảng A2 (V ≤ 20 m/s: 2,1·10⁻⁶)</t>
+          <t>Bảng 9, theo α</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="36" t="inlineStr">
         <is>
-          <t>Độ dềnh do gió Δh</t>
+          <t>Chiều cao sóng leo hsl1%</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
@@ -3472,113 +3499,191 @@
           <t>m</t>
         </is>
       </c>
-      <c r="C33" s="38">
-        <f>C32*C10^2*C12/(g_*C7)*COS(RADIANS(C11))</f>
-        <v/>
-      </c>
-      <c r="D33" s="38">
-        <f>D32*D10^2*D12/(g_*D7)*COS(RADIANS(D11))</f>
-        <v/>
-      </c>
-      <c r="E33" s="38">
-        <f>E32*E10^2*E12/(g_*E7)*COS(RADIANS(E11))</f>
-        <v/>
-      </c>
-      <c r="F33" s="38">
-        <f>F32*F10^2*F12/(g_*F7)*COS(RADIANS(F11))</f>
-        <v/>
-      </c>
-      <c r="G33" s="38">
-        <f>G32*G10^2*G12/(g_*G7)*COS(RADIANS(G11))</f>
-        <v/>
-      </c>
-      <c r="H33" s="38">
-        <f>H32*H10^2*H12/(g_*H7)*COS(RADIANS(H11))</f>
+      <c r="C33" s="27">
+        <f>C27*C28*C29*C31*C32*C25</f>
+        <v/>
+      </c>
+      <c r="D33" s="27">
+        <f>D27*D28*D29*D31*D32*D25</f>
+        <v/>
+      </c>
+      <c r="E33" s="27">
+        <f>E27*E28*E29*E31*E32*E25</f>
+        <v/>
+      </c>
+      <c r="F33" s="27">
+        <f>F27*F28*F29*F31*F32*F25</f>
+        <v/>
+      </c>
+      <c r="G33" s="27">
+        <f>G27*G28*G29*G31*G32*G25</f>
+        <v/>
+      </c>
+      <c r="H33" s="27">
+        <f>H27*H28*H29*H31*H32*H25</f>
         <v/>
       </c>
       <c r="I33" s="31" t="inlineStr">
         <is>
-          <t>Δh = kw·V²·D/(g·H)·cos α</t>
+          <t>hsl1% = kr·kp·ksp·krun·kα·h1%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="29" t="inlineStr">
         <is>
-          <t>Độ vượt cao an toàn</t>
-        </is>
-      </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="C34" s="32">
-        <f>IF(C5="Z1",a_1,a_2)</f>
-        <v/>
-      </c>
-      <c r="D34" s="32">
-        <f>IF(D5="Z1",a_1,a_2)</f>
-        <v/>
-      </c>
-      <c r="E34" s="32">
-        <f>IF(E5="Z1",a_1,a_2)</f>
-        <v/>
-      </c>
-      <c r="F34" s="32">
-        <f>IF(F5="Z1",a_1,a_2)</f>
-        <v/>
-      </c>
-      <c r="G34" s="32">
-        <f>IF(G5="Z1",a_1,a_2)</f>
-        <v/>
-      </c>
-      <c r="H34" s="32">
-        <f>IF(H5="Z1",a_1,a_2)</f>
+          <t>Hệ số kw</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr"/>
+      <c r="C34" s="37">
+        <f>IF(C10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(C10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(C10,KW_V,1))+(C10-INDEX(KW_V,MATCH(C10,KW_V,1)))*(INDEX(KW_k,MATCH(C10,KW_V,1)+1)-INDEX(KW_k,MATCH(C10,KW_V,1)))/(INDEX(KW_V,MATCH(C10,KW_V,1)+1)-INDEX(KW_V,MATCH(C10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="D34" s="37">
+        <f>IF(D10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(D10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(D10,KW_V,1))+(D10-INDEX(KW_V,MATCH(D10,KW_V,1)))*(INDEX(KW_k,MATCH(D10,KW_V,1)+1)-INDEX(KW_k,MATCH(D10,KW_V,1)))/(INDEX(KW_V,MATCH(D10,KW_V,1)+1)-INDEX(KW_V,MATCH(D10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="E34" s="37">
+        <f>IF(E10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(E10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(E10,KW_V,1))+(E10-INDEX(KW_V,MATCH(E10,KW_V,1)))*(INDEX(KW_k,MATCH(E10,KW_V,1)+1)-INDEX(KW_k,MATCH(E10,KW_V,1)))/(INDEX(KW_V,MATCH(E10,KW_V,1)+1)-INDEX(KW_V,MATCH(E10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="F34" s="37">
+        <f>IF(F10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(F10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(F10,KW_V,1))+(F10-INDEX(KW_V,MATCH(F10,KW_V,1)))*(INDEX(KW_k,MATCH(F10,KW_V,1)+1)-INDEX(KW_k,MATCH(F10,KW_V,1)))/(INDEX(KW_V,MATCH(F10,KW_V,1)+1)-INDEX(KW_V,MATCH(F10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="G34" s="37">
+        <f>IF(G10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(G10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(G10,KW_V,1))+(G10-INDEX(KW_V,MATCH(G10,KW_V,1)))*(INDEX(KW_k,MATCH(G10,KW_V,1)+1)-INDEX(KW_k,MATCH(G10,KW_V,1)))/(INDEX(KW_V,MATCH(G10,KW_V,1)+1)-INDEX(KW_V,MATCH(G10,KW_V,1)))))</f>
+        <v/>
+      </c>
+      <c r="H34" s="37">
+        <f>IF(H10&lt;=INDEX(KW_V,1),INDEX(KW_k,1),IF(H10&gt;=INDEX(KW_V,COUNT(KW_V)),INDEX(KW_k,COUNT(KW_V)),INDEX(KW_k,MATCH(H10,KW_V,1))+(H10-INDEX(KW_V,MATCH(H10,KW_V,1)))*(INDEX(KW_k,MATCH(H10,KW_V,1)+1)-INDEX(KW_k,MATCH(H10,KW_V,1)))/(INDEX(KW_V,MATCH(H10,KW_V,1)+1)-INDEX(KW_V,MATCH(H10,KW_V,1)))))</f>
         <v/>
       </c>
       <c r="I34" s="31" t="inlineStr">
         <is>
-          <t>a (Z1), a′ (Z2) – Bảng 3</t>
+          <t>Bảng A2 (V ≤ 20 m/s: 2,1·10⁻⁶)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="36" t="inlineStr">
         <is>
+          <t>Độ dềnh do gió Δh</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C35" s="38">
+        <f>C34*C10^2*C12/(g_*C7)*COS(RADIANS(C11))</f>
+        <v/>
+      </c>
+      <c r="D35" s="38">
+        <f>D34*D10^2*D12/(g_*D7)*COS(RADIANS(D11))</f>
+        <v/>
+      </c>
+      <c r="E35" s="38">
+        <f>E34*E10^2*E12/(g_*E7)*COS(RADIANS(E11))</f>
+        <v/>
+      </c>
+      <c r="F35" s="38">
+        <f>F34*F10^2*F12/(g_*F7)*COS(RADIANS(F11))</f>
+        <v/>
+      </c>
+      <c r="G35" s="38">
+        <f>G34*G10^2*G12/(g_*G7)*COS(RADIANS(G11))</f>
+        <v/>
+      </c>
+      <c r="H35" s="38">
+        <f>H34*H10^2*H12/(g_*H7)*COS(RADIANS(H11))</f>
+        <v/>
+      </c>
+      <c r="I35" s="31" t="inlineStr">
+        <is>
+          <t>Δh = kw·V²·D/(g·H)·cos α</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="inlineStr">
+        <is>
+          <t>Độ vượt cao an toàn</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="C36" s="32">
+        <f>IF(C5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="D36" s="32">
+        <f>IF(D5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="E36" s="32">
+        <f>IF(E5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="F36" s="32">
+        <f>IF(F5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="G36" s="32">
+        <f>IF(G5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="H36" s="32">
+        <f>IF(H5="Z1",a_1,a_2)</f>
+        <v/>
+      </c>
+      <c r="I36" s="31" t="inlineStr">
+        <is>
+          <t>a (Z1), a′ (Z2) – Bảng 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="36" t="inlineStr">
+        <is>
           <t>Cao trình đỉnh đập yêu cầu Z₁ hoặc Z₂</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="C35" s="39">
-        <f>C6+C33+C31+C34</f>
-        <v/>
-      </c>
-      <c r="D35" s="39">
-        <f>D6+D33+D31+D34</f>
-        <v/>
-      </c>
-      <c r="E35" s="39">
-        <f>E6+E33+E31+E34</f>
-        <v/>
-      </c>
-      <c r="F35" s="39">
-        <f>F6+F33+F31+F34</f>
-        <v/>
-      </c>
-      <c r="G35" s="39">
-        <f>G6+G33+G31+G34</f>
-        <v/>
-      </c>
-      <c r="H35" s="39">
-        <f>H6+H33+H31+H34</f>
-        <v/>
-      </c>
-      <c r="I35" s="31" t="inlineStr">
+      <c r="C37" s="39">
+        <f>C6+C35+C33+C36</f>
+        <v/>
+      </c>
+      <c r="D37" s="39">
+        <f>D6+D35+D33+D36</f>
+        <v/>
+      </c>
+      <c r="E37" s="39">
+        <f>E6+E35+E33+E36</f>
+        <v/>
+      </c>
+      <c r="F37" s="39">
+        <f>F6+F35+F33+F36</f>
+        <v/>
+      </c>
+      <c r="G37" s="39">
+        <f>G6+G35+G33+G36</f>
+        <v/>
+      </c>
+      <c r="H37" s="39">
+        <f>H6+H35+H33+H36</f>
+        <v/>
+      </c>
+      <c r="I37" s="31" t="inlineStr">
         <is>
           <t>Z = Z + Δh + hsl + a</t>
         </is>
@@ -3702,7 +3807,7 @@
         <v/>
       </c>
       <c r="C6" s="32">
-        <f>TinhSong!C30</f>
+        <f>TinhSong!C32</f>
         <v/>
       </c>
       <c r="D6" s="32">
@@ -3714,19 +3819,19 @@
         <v/>
       </c>
       <c r="F6" s="34">
-        <f>TinhSong!C31</f>
+        <f>TinhSong!C33</f>
         <v/>
       </c>
       <c r="G6" s="34">
-        <f>TinhSong!D31</f>
+        <f>TinhSong!D33</f>
         <v/>
       </c>
       <c r="H6" s="40">
-        <f>TinhSong!C35</f>
+        <f>TinhSong!C37</f>
         <v/>
       </c>
       <c r="I6" s="40">
-        <f>TinhSong!D35</f>
+        <f>TinhSong!D37</f>
         <v/>
       </c>
       <c r="J6" s="40">
@@ -3749,7 +3854,7 @@
         <v/>
       </c>
       <c r="C7" s="32">
-        <f>TinhSong!E30</f>
+        <f>TinhSong!E32</f>
         <v/>
       </c>
       <c r="D7" s="32">
@@ -3761,19 +3866,19 @@
         <v/>
       </c>
       <c r="F7" s="34">
-        <f>TinhSong!E31</f>
+        <f>TinhSong!E33</f>
         <v/>
       </c>
       <c r="G7" s="34">
-        <f>TinhSong!F31</f>
+        <f>TinhSong!F33</f>
         <v/>
       </c>
       <c r="H7" s="40">
-        <f>TinhSong!E35</f>
+        <f>TinhSong!E37</f>
         <v/>
       </c>
       <c r="I7" s="40">
-        <f>TinhSong!F35</f>
+        <f>TinhSong!F37</f>
         <v/>
       </c>
       <c r="J7" s="40">
@@ -3796,7 +3901,7 @@
         <v/>
       </c>
       <c r="C8" s="32">
-        <f>TinhSong!G30</f>
+        <f>TinhSong!G32</f>
         <v/>
       </c>
       <c r="D8" s="32">
@@ -3808,19 +3913,19 @@
         <v/>
       </c>
       <c r="F8" s="34">
-        <f>TinhSong!G31</f>
+        <f>TinhSong!G33</f>
         <v/>
       </c>
       <c r="G8" s="34">
-        <f>TinhSong!H31</f>
+        <f>TinhSong!H33</f>
         <v/>
       </c>
       <c r="H8" s="40">
-        <f>TinhSong!G35</f>
+        <f>TinhSong!G37</f>
         <v/>
       </c>
       <c r="I8" s="40">
-        <f>TinhSong!H35</f>
+        <f>TinhSong!H37</f>
         <v/>
       </c>
       <c r="J8" s="40">
@@ -4256,12 +4361,12 @@
         </is>
       </c>
       <c r="B32" s="32">
-        <f>TinhSong!C22</f>
+        <f>TinhSong!C24</f>
         <v/>
       </c>
       <c r="C32" s="11" t="n"/>
       <c r="D32" s="32">
-        <f>TinhSong!D22</f>
+        <f>TinhSong!D24</f>
         <v/>
       </c>
       <c r="E32" s="11" t="n"/>
@@ -4278,12 +4383,12 @@
         </is>
       </c>
       <c r="B33" s="34">
-        <f>TinhSong!C23</f>
+        <f>TinhSong!C25</f>
         <v/>
       </c>
       <c r="C33" s="11" t="n"/>
       <c r="D33" s="34">
-        <f>TinhSong!D23</f>
+        <f>TinhSong!D25</f>
         <v/>
       </c>
       <c r="E33" s="11" t="n"/>
@@ -4300,12 +4405,12 @@
         </is>
       </c>
       <c r="B34" s="32">
-        <f>TinhSong!C25</f>
+        <f>TinhSong!C27</f>
         <v/>
       </c>
       <c r="C34" s="11" t="n"/>
       <c r="D34" s="32">
-        <f>TinhSong!D25</f>
+        <f>TinhSong!D27</f>
         <v/>
       </c>
       <c r="E34" s="11" t="n"/>
@@ -4322,12 +4427,12 @@
         </is>
       </c>
       <c r="B35" s="32">
-        <f>TinhSong!C26</f>
+        <f>TinhSong!C28</f>
         <v/>
       </c>
       <c r="C35" s="11" t="n"/>
       <c r="D35" s="32">
-        <f>TinhSong!D26</f>
+        <f>TinhSong!D28</f>
         <v/>
       </c>
       <c r="E35" s="11" t="n"/>
@@ -4344,12 +4449,12 @@
         </is>
       </c>
       <c r="B36" s="32">
-        <f>TinhSong!C27</f>
+        <f>TinhSong!C29</f>
         <v/>
       </c>
       <c r="C36" s="11" t="n"/>
       <c r="D36" s="32">
-        <f>TinhSong!D27</f>
+        <f>TinhSong!D29</f>
         <v/>
       </c>
       <c r="E36" s="11" t="n"/>
@@ -4366,12 +4471,12 @@
         </is>
       </c>
       <c r="B37" s="32">
-        <f>TinhSong!C29</f>
+        <f>TinhSong!C31</f>
         <v/>
       </c>
       <c r="C37" s="11" t="n"/>
       <c r="D37" s="32">
-        <f>TinhSong!D29</f>
+        <f>TinhSong!D31</f>
         <v/>
       </c>
       <c r="E37" s="11" t="n"/>
@@ -4388,12 +4493,12 @@
         </is>
       </c>
       <c r="B38" s="32">
-        <f>TinhSong!C30</f>
+        <f>TinhSong!C32</f>
         <v/>
       </c>
       <c r="C38" s="11" t="n"/>
       <c r="D38" s="32">
-        <f>TinhSong!D30</f>
+        <f>TinhSong!D32</f>
         <v/>
       </c>
       <c r="E38" s="11" t="n"/>
@@ -4410,12 +4515,12 @@
         </is>
       </c>
       <c r="B39" s="34">
-        <f>TinhSong!C31</f>
+        <f>TinhSong!C33</f>
         <v/>
       </c>
       <c r="C39" s="11" t="n"/>
       <c r="D39" s="34">
-        <f>TinhSong!D31</f>
+        <f>TinhSong!D33</f>
         <v/>
       </c>
       <c r="E39" s="11" t="n"/>
@@ -4432,12 +4537,12 @@
         </is>
       </c>
       <c r="B40" s="34">
-        <f>TinhSong!C33</f>
+        <f>TinhSong!C35</f>
         <v/>
       </c>
       <c r="C40" s="11" t="n"/>
       <c r="D40" s="34">
-        <f>TinhSong!D33</f>
+        <f>TinhSong!D35</f>
         <v/>
       </c>
       <c r="E40" s="11" t="n"/>
@@ -4454,12 +4559,12 @@
         </is>
       </c>
       <c r="B41" s="32">
-        <f>TinhSong!C34</f>
+        <f>TinhSong!C36</f>
         <v/>
       </c>
       <c r="C41" s="11" t="n"/>
       <c r="D41" s="32">
-        <f>TinhSong!D34</f>
+        <f>TinhSong!D36</f>
         <v/>
       </c>
       <c r="E41" s="11" t="n"/>
@@ -4475,12 +4580,12 @@
         </is>
       </c>
       <c r="B42" s="43">
-        <f>TinhSong!C35</f>
+        <f>TinhSong!C37</f>
         <v/>
       </c>
       <c r="C42" s="11" t="n"/>
       <c r="D42" s="43">
-        <f>TinhSong!D35</f>
+        <f>TinhSong!D37</f>
         <v/>
       </c>
       <c r="E42" s="11" t="n"/>

</xml_diff>